<commit_message>
Corrige les URLs images cassees (Parsons/photo cpersons->cparsons, Bourgeois extension manquante, Gosala nom de fichier)
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-france.xlsx
+++ b/data/frise-philosophes-france.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Philosophes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Mode_d_emploi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Philosophes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mode_d_emploi" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Philosophes'!$A$3:$I$138</definedName>
@@ -896,7 +896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M141"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4.59" customWidth="1" style="44" min="1" max="1"/>
@@ -1680,7 +1680,7 @@
       <c r="F16" s="57" t="n"/>
       <c r="G16" s="63" t="inlineStr">
         <is>
-          <t>
+          <t xml:space="preserve">
 </t>
         </is>
       </c>
@@ -1790,7 +1790,7 @@
       <c r="F18" s="57" t="n"/>
       <c r="G18" s="63" t="inlineStr">
         <is>
-          <t>
+          <t xml:space="preserve">
 </t>
         </is>
       </c>
@@ -7008,7 +7008,7 @@
       </c>
       <c r="H114" s="62" t="inlineStr">
         <is>
-          <t>https://www.laphilo.fr/pho/bbourgeois-mini</t>
+          <t>https://www.laphilo.fr/pho/bbourgeois-mini.webp</t>
         </is>
       </c>
       <c r="J114" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Distingue les descriptions de 9 philosophes qui partageaient la même
Ammonios Saccas portait par erreur la description de Speusippe (« neveu
de Platon ») : il est le maître de Plotin. Milhaud/Rey, Hégésinous/
Téléclès, Boèce/Cassiodore et Ogniov/Boldyrev ont chacun la leur.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-france.xlsx
+++ b/data/frise-philosophes-france.xlsx
@@ -2551,7 +2551,7 @@
       </c>
       <c r="L31" s="48" t="inlineStr">
         <is>
-          <t>philosophe français spécialiste d'histoire et de philosophie des sciences.</t>
+          <t>philosophe français des sciences, pionnier du conventionnalisme et spécialiste des fondements de la géométrie.</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="L47" s="48" t="inlineStr">
         <is>
-          <t>philosophe français spécialiste d'histoire et de philosophie des sciences.</t>
+          <t>philosophe français, historien des sciences et cofondateur de l'Institut d'histoire des sciences en 1932.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dates corrigées d'après Wikidata et Wikipédia : Grosseteste (mort en 1253), Sextus Empiricus (vers 160 – vers 210 apr. J.-C.), Xunzi (vers 310 – 235 av. J.-C.), Dharmakirti (vers 600 – 660), Pierre d'Ailly (mort en 1420), Morot-Sir (mort en 1993), Théophraste (vers 372 – 288 av. J.-C.), Leśniewski (né en 1886), Vine Deloria Jr. (né en 1933) ; Éliane Escoubas, morte le 18 juillet 2026 : date de décès, texte, fiche déplacée de france-actif vers france
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-france.xlsx
+++ b/data/frise-philosophes-france.xlsx
@@ -938,7 +938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O153"/>
+  <dimension ref="A1:O154"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4.59" customWidth="1" style="47" min="1" max="1"/>
@@ -6125,15 +6125,15 @@
       </c>
     </row>
     <row r="88" ht="162" customHeight="1" s="49">
-      <c r="A88" s="57" t="n">
+      <c r="A88" s="57">
         <v>1910</v>
       </c>
-      <c r="B88" s="57" t="n">
-        <v>1999</v>
+      <c r="B88" s="57">
+        <v>1993</v>
       </c>
       <c r="C88" s="60" t="inlineStr">
         <is>
-          <t>1910 – 1999</t>
+          <t xml:space="preserve">1910 – 1993</t>
         </is>
       </c>
       <c r="D88" s="60" t="inlineStr">
@@ -10036,6 +10036,65 @@
         </is>
       </c>
       <c r="O153"/>
+    </row>
+    <row r="154" ht="176.25" customHeight="1" s="49">
+      <c r="A154" s="47">
+        <v>1937</v>
+      </c>
+      <c r="B154" s="47">
+        <v>2026</v>
+      </c>
+      <c r="C154" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1937 – 2026</t>
+        </is>
+      </c>
+      <c r="D154" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Éliane ESCOUBAS</t>
+        </is>
+      </c>
+      <c r="E154" s="85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89liane_Escoubas"  style="color:#6A142A"  title=" Wikipedia"&gt;Éliane ESCOUBAS&lt;/a&gt;  est une philosophe française, historienne de la philosophie et traductrice. Elle se rattache à l’école phénoménologique et travaille principalement sur la philosophie allemande, la phénoménologie de l’art et la psychiatrie phénoménologique, dite Daseinsanalyse. Après une formation marquée par les cours de Gérard Granel sur Husserl, Kant et Hegel à Toulouse, elle enseigne dans le secondaire puis devient maître de conférences, puis professeur de philosophie, tout en menant des recherches au CNRS et en participant à la création du Collège international de Philosophie. &lt;/p&gt; &lt;p&gt; Elle met au centre la phénoménologie de l’expérience sensible, en particulier la manière dont le monde et le sujet adviennent à travers le sentir, l’affect et la perception. Elle montre que la phénoménologie fournit un prisme particulièrement adapté pour penser l’esthétique, car l’œuvre d’art apparaît comme un mode privilégié pour saisir comment le sujet et le monde se co‑constituent dans une expérience sensible et existentielle. &lt;/p&gt; &lt;p&gt; Une grande partie de son œuvre est consacrée à une « esthétique du sentir » où l’art n’est pas seulement une illustration de la philosophie, mais un mode de connaissance autonome. Dans ses travaux comme Imago mundi. Topologie de l’art ou L’invention de l’art, elle montre que l’image et l’œuvre picturale ne se réduisent pas à « représentation » ou « signe », mais relèvent d’une apparition du monde lui‑même, d’une spatialité et d’une temporalité qui précèdent les catégories classiques de l’objet. &lt;/p&gt; &lt;p&gt; Sa philosophie s’ouvre aussi à la phénoménologie clinique et à la psychiatrie, notamment à travers la Daseinsanalyse et la place de l’affect et de l’affectivité dans la constitution du sujet. En explorant les affectivités dans la modernité et la phénoménologie, Escoubas prolonge ainsi une réflexion sur la manière dont le vécu, le corps et la subjectivité forment un champ de savoir propre, à la fois esthétique, analytique et existentiel. Elle meurt à Paris le 18 juillet 2026. &lt;/p&gt;  &lt;audio controls title="Alain BADIOU par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10080-25.11.2011-ITEMA_20320112-2011C3403E0190-ITE_00047070_RSCE-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
+</t>
+        </is>
+      </c>
+      <c r="H154" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/eescoubas-mini.webp</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://laphilo.fr/photo/escoubas.webp</t>
+        </is>
+      </c>
+      <c r="J154" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">esthetique ; epistemologie</t>
+        </is>
+      </c>
+      <c r="K154" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénoménologie</t>
+        </is>
+      </c>
+      <c r="L154" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe française, historienne de la philosophie et traductrice.</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">femme</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
     </row>
     <row r="1048566" ht="12.75" customHeight="1" s="49"/>
     <row r="1048567" ht="12.75" customHeight="1" s="49"/>

</xml_diff>

<commit_message>
Refonte de /histoire-des-philosophes/ et de /histoire-des-courants/ en sept traditions (Proche-Orient ancien, Occident par époques, Inde, Asie de l'Est, Islam et pensée juive, Russie, Afrique et Amériques), sommaire visible sur ordinateur
Histoire des philosophes : 26 cartouches (18 renommés ; Contemporains scindé en XIXe et XXe siècle ; 6 nouveaux : Proche-Orient ancien, Inde moderne, Corée, islam moderne, Russie, Amériques et Caraïbes) ; doublons retirés (Boèce, Spinoza, Byung-Chul Han), Foucault au XXe siècle, Imhotep, Césaire et Fanon déplacés ; erreurs corrigées (triade de Fichte, flatus vocis, Nicolas de Cues, Machiavel, Averroès et la double vérité, al-Kindi, Ibn Khaldoun, Nishida) ; page renommée « L'histoire des philosophes » (accueil, bienvenue, llms.txt).
Fiche « Mohammed Abed AL-JABRI » (était « Mohamed Abel ») avec 301 depuis l'ancienne adresse ; titre du podcast d'Éliane Escoubas (correction de l'éditeur).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/frise-philosophes-france.xlsx
+++ b/data/frise-philosophes-france.xlsx
@@ -8550,1016 +8550,1021 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="185.25" customHeight="1" s="49">
-      <c r="A128" s="57" t="n">
+    <row r="128" ht="176.25" customHeight="1" s="49">
+      <c r="A128" s="47">
+        <v>1937</v>
+      </c>
+      <c r="B128" s="47">
+        <v>2026</v>
+      </c>
+      <c r="C128" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1937 – 2026</t>
+        </is>
+      </c>
+      <c r="D128" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Éliane ESCOUBAS</t>
+        </is>
+      </c>
+      <c r="E128" s="85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89liane_Escoubas"  style="color:#6A142A"  title=" Wikipedia"&gt;Éliane ESCOUBAS&lt;/a&gt;  est une philosophe française, historienne de la philosophie et traductrice. Elle se rattache à l’école phénoménologique et travaille principalement sur la philosophie allemande, la phénoménologie de l’art et la psychiatrie phénoménologique, dite Daseinsanalyse. Après une formation marquée par les cours de Gérard Granel sur Husserl, Kant et Hegel à Toulouse, elle enseigne dans le secondaire puis devient maître de conférences, puis professeur de philosophie, tout en menant des recherches au CNRS et en participant à la création du Collège international de Philosophie. &lt;/p&gt; &lt;p&gt; Elle met au centre la phénoménologie de l’expérience sensible, en particulier la manière dont le monde et le sujet adviennent à travers le sentir, l’affect et la perception. Elle montre que la phénoménologie fournit un prisme particulièrement adapté pour penser l’esthétique, car l’œuvre d’art apparaît comme un mode privilégié pour saisir comment le sujet et le monde se co‑constituent dans une expérience sensible et existentielle. &lt;/p&gt; &lt;p&gt; Une grande partie de son œuvre est consacrée à une « esthétique du sentir » où l’art n’est pas seulement une illustration de la philosophie, mais un mode de connaissance autonome. Dans ses travaux comme Imago mundi. Topologie de l’art ou L’invention de l’art, elle montre que l’image et l’œuvre picturale ne se réduisent pas à « représentation » ou « signe », mais relèvent d’une apparition du monde lui‑même, d’une spatialité et d’une temporalité qui précèdent les catégories classiques de l’objet. &lt;/p&gt; &lt;p&gt; Sa philosophie s’ouvre aussi à la phénoménologie clinique et à la psychiatrie, notamment à travers la Daseinsanalyse et la place de l’affect et de l’affectivité dans la constitution du sujet. En explorant les affectivités dans la modernité et la phénoménologie, Escoubas prolonge ainsi une réflexion sur la manière dont le vécu, le corps et la subjectivité forment un champ de savoir propre, à la fois esthétique, analytique et existentiel. Elle meurt à Paris le 18 juillet 2026. &lt;/p&gt;  &lt;audio controls title="Eliane ESCOUBAS par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10080-25.11.2011-ITEMA_20320112-2011C3403E0190-ITE_00047070_RSCE-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
+      </c>
+      <c r="H128" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/eescoubas-mini.webp</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://laphilo.fr/photo/escoubas.webp</t>
+        </is>
+      </c>
+      <c r="J128" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">esthetique ; epistemologie</t>
+        </is>
+      </c>
+      <c r="K128" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phénoménologie</t>
+        </is>
+      </c>
+      <c r="L128" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">philosophe française, historienne de la philosophie et traductrice.</t>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">femme</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="185.25" customHeight="1" s="49">
+      <c r="A129" s="57" t="n">
         <v>1938</v>
       </c>
-      <c r="B128" s="57" t="inlineStr">
+      <c r="B129" s="57" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="C128" s="57" t="inlineStr">
+      <c r="C129" s="57" t="inlineStr">
         <is>
           <t>1938 – 2017</t>
         </is>
       </c>
-      <c r="D128" s="58" t="inlineStr">
+      <c r="D129" s="58" t="inlineStr">
         <is>
           <t>Jean-François MARQUET</t>
         </is>
       </c>
-      <c r="E128" s="59" t="inlineStr">
+      <c r="E129" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jean-Fran%C3%A7ois_Marquet"  title=" Wikipedia"&gt;Jean-François MARQUET&lt;/a&gt; était un philosophe français spécialiste de l'idéalisme allemand et de la mystique, connu pour ses travaux sur Schelling, Hegel, Böhme et &lt;a href="https://fr.wikipedia.org/wiki/N%C3%A9oplatonisme"  title=" neoplatonisme par Wikipedia"&gt;le néoplatonisme. &lt;/a&gt; Agrégé de philosophie et professeur à l'Université Paris-Sorbonne, il fut l'un des meilleurs connaisseurs français de Schelling et l'un des rares philosophes à s'être intéressé aux connexions entre la philosophie spéculative allemande et les traditions mystiques occidentales. &lt;/p&gt; &lt;p&gt; Sa thèse principale, &lt;em&gt;Liberté et Existence. Étude sur la formation de la philosophie de Schelling&lt;/em&gt; (1973), est une analyse rigoureuse et pénétrante du développement de la pensée de Schelling, depuis les premiers textes influencés par Fichte jusqu'à la philosophie tardive de la liberté et de la mythologie. Il y montre la cohérence profonde d'une pensée souvent jugée dispersée, en la centrant sur la problématique de la liberté comme indifférence originaire de l'être. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Miroirs de l'identité. La Littérature hantée par la philosophie&lt;/em&gt; (1996), il explore les relations entre philosophie et littérature à travers des auteurs comme Novalis, Kleist, Hoffmann et Nerval. Ses études sur Jakob Böhme et les thiosophes germaniques contribuèrent à ouvrir la philosophie française à des courants méconnus mais essentiels pour comprendre l'émergence de l'idéalisme allemand. Il représente un philosophe  &lt;a href="https://www.persee.fr/doc/abpo_0399-0826_1976_num_83_2_2819"  title=" les calendriers positivistes par persée"&gt;d'une rare érudition, &lt;/a&gt; capable de naviguer entre la rigueur conceptuelle et l'ouverture aux dimensions poétiques et spirituelles de la pensée. &lt;/p&gt;  &lt;audio controls title="Les strategies du secret par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10194-14.02.2007-ITEMA_20058582-2007C3035S0033-MEM_000035816_RF-21.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  </t>
         </is>
       </c>
-      <c r="F128" s="57" t="inlineStr">
+      <c r="F129" s="57" t="inlineStr">
         <is>
           <t>W1PdYExCQRY</t>
         </is>
       </c>
-      <c r="G128" s="59" t="inlineStr">
+      <c r="G129" s="59" t="inlineStr">
         <is>
           <t>"JEAN FRANCOIS MARQUET" par Didier Doc Pilot</t>
         </is>
       </c>
-      <c r="H128" s="65" t="inlineStr">
+      <c r="H129" s="65" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/jfmarquet-mini.webp</t>
         </is>
       </c>
-      <c r="J128" s="48" t="inlineStr">
+      <c r="J129" s="48" t="inlineStr">
         <is>
           <t>metaphysique</t>
         </is>
       </c>
-      <c r="K128" s="48" t="inlineStr">
+      <c r="K129" s="48" t="inlineStr">
         <is>
           <t>Phénoménologie</t>
         </is>
       </c>
-      <c r="L128" s="48" t="inlineStr">
+      <c r="L129" s="48" t="inlineStr">
         <is>
           <t>philosophe français spécialiste de l'idéalisme allemand et de la mystique.</t>
         </is>
       </c>
-      <c r="N128" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="216.75" customHeight="1" s="49">
-      <c r="A129" s="54" t="n">
+      <c r="N129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="216.75" customHeight="1" s="49">
+      <c r="A130" s="54" t="n">
         <v>1939</v>
       </c>
-      <c r="B129" s="54" t="inlineStr">
+      <c r="B130" s="54" t="inlineStr">
         <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="C129" s="54" t="inlineStr">
+      <c r="C130" s="54" t="inlineStr">
         <is>
           <t>1939 – 2018</t>
         </is>
       </c>
-      <c r="D129" s="55" t="inlineStr">
+      <c r="D130" s="55" t="inlineStr">
         <is>
           <t>Clément ROSSET</t>
         </is>
       </c>
-      <c r="E129" s="62" t="inlineStr">
+      <c r="E130" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Cl%C3%A9ment_Rosset" title=" Wikipedia"&gt;Clément ROSSET&lt;/a&gt; était un philosophe français connu pour sa pensée radicale et son style d'écriture d'une grande clarté. Son œuvre est principalement centrée sur le concept du  &lt;a href="https://www.youtube.com/watch?v=I50Jbj6uQEU" title="Clément Rosset : la réalité ne convient pas ! par Kosmos"&gt;"réel"&lt;/a&gt;  et l'incapacité ou la difficulté de l'homme à l'accepter dans sa singularité et souvent sa cruauté. &lt;/p&gt; &lt;p&gt;&lt;a href="https://www.youtube.com/watch?v=8m_kXVBdtwg"  title=" Le réel et son double, Clément Rosset, 2.2 avant-propos par Thibault BELZACQ"&gt;Le Réel sans double&lt;/a&gt; : Son idée maîtresse est que le réel est unique, singulier et dépourvu de tout "double". Il n'y a pas d'arrière-monde, pas de sens caché, pas de consolation ou d'illusion qui puisse atténuer sa nature brute. Le réel est simplement ce qui est, dans son évidence la plus nue. &lt;/p&gt; &lt;p&gt;Le Refus du double et de l'illusion : Une grande partie de son travail consiste à traquer les différentes formes d'illusions et de doubles que l'humanité crée pour  &lt;a href="https://philitt.fr/2023/09/12/clement-rosset-tout-est-sans-raison/"  title="Clément Rosset : tout est sans raison par Phillitt"&gt;échapper à la confrontation&lt;/a&gt; directe avec le réel. Ces doubles peuvent être d'ordre métaphysique, moral, psychologique, ou même esthétique.&lt;/p&gt; &lt;p&gt;&lt;a href="https://www.youtube.com/watch?v=JDcudFE_uBQ"  title="Entretien avec Pierre Dumayet (1961) par Archives"&gt;Philosophie tragique&lt;/a&gt; et Joie : Bien que sa pensée puisse sembler sombre en insistant sur la cruauté et l'absurdité du réel, il développe une philosophie que l'on qualifie souvent de "tragique" au sens nietzschéen du terme. Il ne s'agit pas de désespoir, mais plutôt de l'affirmation de la vie et du réel tels qu'ils sont, y compris dans leurs aspects les plus difficiles. &lt;/p&gt; &lt;p&gt; Il est également remarquable par son style d'écriture. Loin du jargon philosophique abscons, il privilégie une langue simple, directe et percutante. Cette clarté formelle est au service de la clarté de sa pensée, cherchant à énoncer le réel avec le moins d'interférences possible. Son œuvre, bien que parfois restée en marge des courants universitaires dominants, a marqué par sa radicalité, sa lucidité et sa défense d'une confrontation sans fard avec le réel.  &lt;/p&gt; &lt;audio controls title="Clément Rosset par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10080-20.12.2013-ITEMA_20564152-2013C3403E0215-21.mp3" type="audio/mpeg" align="center"&gt;&lt;/audio&gt;  </t>
         </is>
       </c>
-      <c r="F129" s="54" t="inlineStr">
+      <c r="F130" s="54" t="inlineStr">
         <is>
           <t>9m6CPt4pRlw</t>
         </is>
       </c>
-      <c r="G129" s="56" t="inlineStr">
+      <c r="G130" s="56" t="inlineStr">
         <is>
           <t>"Clément Rosset (1): Heureux, malgré tout" par Camille Tassel</t>
         </is>
       </c>
-      <c r="H129" s="62" t="inlineStr">
+      <c r="H130" s="62" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/rosset-mini.webp</t>
         </is>
       </c>
-      <c r="J129" s="48" t="inlineStr">
+      <c r="J130" s="48" t="inlineStr">
         <is>
           <t>metaphysique ; ethique</t>
         </is>
       </c>
-      <c r="K129" s="48" t="inlineStr">
+      <c r="K130" s="48" t="inlineStr">
         <is>
           <t>Naturalisme</t>
         </is>
       </c>
-      <c r="L129" s="48" t="inlineStr">
+      <c r="L130" s="48" t="inlineStr">
         <is>
           <t>philosophe français du tragique et de la théorie du réel.</t>
         </is>
       </c>
-      <c r="N129" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="199.5" customHeight="1" s="49">
-      <c r="A130" s="57" t="n">
+      <c r="N130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="199.5" customHeight="1" s="49">
+      <c r="A131" s="57" t="n">
         <v>1940</v>
       </c>
-      <c r="B130" s="57" t="inlineStr">
+      <c r="B131" s="57" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C130" s="57" t="inlineStr">
+      <c r="C131" s="57" t="inlineStr">
         <is>
           <t>1940 – 2021</t>
         </is>
       </c>
-      <c r="D130" s="58" t="inlineStr">
+      <c r="D131" s="58" t="inlineStr">
         <is>
           <t>Jacques BOUVERESSE</t>
         </is>
       </c>
-      <c r="E130" s="65" t="inlineStr">
+      <c r="E131" s="65" t="inlineStr">
         <is>
           <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jacques_Bouveresse"  title=" Wikipedia"&gt;Jacques BOUVERESSE&lt;/a&gt; était un philosophe français du courant analytique, connu pour son rationalisme exigeant, son &lt;a href="https://www.youtube.com/watch?v=mfGM00nmj20"  title=" Wittgenstein et l'intériorité 一 Jacques Bouveresse par Andrea Cirla "&gt;travail sur Wittgenstein &lt;/a&gt; et sa critique des dérives du milieu intellectuel français. Il a largement contribué à introduire et stabiliser en France une philosophie soucieuse de vérité, de clarté et d’argumentation rigoureuse. &lt;/p&gt; &lt;p&gt; Ses domaines privilégiés sont la philosophie de la connaissance, des sciences, des mathématiques, de la logique, du langage, ainsi qu’une philosophie de la culture attentive à la littérature et à la critique sociale.  Il se réclame du rationalisme des Lumières et s’inspire fortement de la philosophie analytique, du Cercle de Vienne, de Frege, de Gödel et de la tradition d’Europe centrale. Wittgenstein, qu’il contribue à faire connaître en France, est l’une de ses références centrales. &lt;/p&gt; &lt;p&gt; Il défend une position rationaliste dont le prolongement éthique est ce qu’il appelle la  &lt;a href="https://www.persee.fr/doc/lgge_0458-726x_1971_num_6_21_2079" title="Langage ordinaire et philosophie par Persée "&gt;"modestie intellectuelle" &lt;/a&gt; : ne pas exagérer ce que la philosophie peut faire, refuser le pathos et le prestige facile. Il combat le relativisme, l’historicisme radical et les remises en cause globales de la notion de vérité, notamment chez certains auteurs français, tout en reconnaissant par ailleurs leur importance. &lt;/p&gt; &lt;p&gt; Sa grande thèse, "Le Mythe de l’intériorité", porte sur Wittgenstein, le langage privé, l’expérience et la signification, et a joué un rôle clé dans la réception française de Wittgenstein. Il consacre de nombreux travaux à Robert Musil et Karl Kraus, qu’il lit comme des alliés dans un combat pour l’exactitude, la critique de la bêtise et des illusions de la culture moderne. &lt;/p&gt;  &lt;audio controls title="Jacques Bouveresse, à la recherche de la clarté par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10351-11.05.2021-ITEMA_23961779-2000C3500E0287-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
-      <c r="F130" s="57" t="inlineStr">
+      <c r="F131" s="57" t="inlineStr">
         <is>
           <t>72_NdVNiFbg</t>
         </is>
       </c>
-      <c r="G130" s="59" t="inlineStr">
+      <c r="G131" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">"Jacques Bouveresse, Prodiges et vertiges de l'analogie" par Philosophie Analytique</t>
         </is>
       </c>
-      <c r="H130" s="65" t="inlineStr">
+      <c r="H131" s="65" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/bouveresse-mini.webp</t>
         </is>
       </c>
-      <c r="J130" s="48" t="inlineStr">
+      <c r="J131" s="48" t="inlineStr">
         <is>
           <t>epistemologie ; logique</t>
         </is>
       </c>
-      <c r="K130" s="48" t="inlineStr">
+      <c r="K131" s="48" t="inlineStr">
         <is>
           <t>Analytique</t>
         </is>
       </c>
-      <c r="L130" s="48" t="inlineStr">
+      <c r="L131" s="48" t="inlineStr">
         <is>
           <t>philosophe français du courant analytique d'un rationalisme exigeant.</t>
         </is>
       </c>
-      <c r="N130" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" ht="164.25" customHeight="1" s="49">
-      <c r="A131" s="54" t="n">
-        <v>1940</v>
-      </c>
-      <c r="B131" s="54" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="C131" s="54" t="inlineStr">
-        <is>
-          <t>1940 – 2021</t>
-        </is>
-      </c>
-      <c r="D131" s="55" t="inlineStr">
-        <is>
-          <t>Jean-Luc NANCY</t>
-        </is>
-      </c>
-      <c r="E131" s="62" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jean-Luc_Nancy"  title=" Wikipedia"&gt;Jean-Luc NANCY&lt;/a&gt; était un philosophe français, agrégé de philosophie, il fut professeur à l'Université de Strasbourg jusqu'à sa retraite. Sa pensée, en dialogue constant avec Heidegger, Derrida et Lacoue-Labarthe — avec lequel il collabora étroitement — porte sur le « sens du monde », la communauté, le corps et le toucher. &lt;/p&gt; &lt;p&gt; Son œuvre est marquée par le questionnement du « with » (avec), du « being-with » heideggerien. Dans &lt;em&gt;La Communauté désoeuvrée&lt;/em&gt; (1986), il développe une pensée de la communauté qui refuse toute forme d'immanentisme ou de fusion : la communauté véritable n'est pas une substance commune, mais  &lt;a href="https://www.youtube.com/watch?v=fZK6pEAPxEw"  title="jean luc Nancy par Institut Humanités "&gt;l'exposition partagée &lt;/a&gt; de la singularité de chacun. Cette réflexion, en dialogue critique avec Blanchot et Bataille, a eu un retentissement considérable dans les débats contemporains sur la politique, la communauté et l'identité. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Corpus&lt;/em&gt; (1992) et &lt;em&gt;Noli me tangere&lt;/em&gt; (2003), il explore  &lt;a href="https://www.youtube.com/watch?v=1kCExw6Wp9k"  title="jean luc Nancy par Lacan TV "&gt;la philosophie du corps &lt;/a&gt; et du toucher comme modes fondamentaux de l'être-au-monde. Son essai sur le sens — &lt;em&gt;Le Sens du monde&lt;/em&gt; (1993) — aborde la question de la possibilité du sens dans un monde déserté par les transcendances. &lt;em&gt;L'Intrus&lt;/em&gt; (2000), bref récit autobiographique sur sa transplantation cardiaque, mêle réflexion philosophique et expérience personnelle de la maladie et de l'altérité. Son œuvre, immense et diverse, témoigne d'une pensée vivante et rigoureuse toujours en dialogue avec la littérature, l'art et la politique. &lt;/p&gt;  &lt;audio controls title="Jean luc Nancy par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/11472-06.02.2011-ITEMA_20267545-2011C16153E0003-ITE_00040439_RSCE-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
-        </is>
-      </c>
-      <c r="F131" s="54" t="inlineStr">
-        <is>
-          <t>0ONnn-EL0BA</t>
-        </is>
-      </c>
-      <c r="G131" s="56" t="inlineStr">
-        <is>
-          <t>"Jean-Luc Nancy, philosophe à l'intelligence sensible" par France Culture</t>
-        </is>
-      </c>
-      <c r="H131" s="62" t="inlineStr">
-        <is>
-          <t>https://www.laphilo.fr/pho/jlnancy-mini.webp</t>
-        </is>
-      </c>
-      <c r="J131" s="48" t="inlineStr">
-        <is>
-          <t>metaphysique ; politique</t>
-        </is>
-      </c>
-      <c r="K131" s="48" t="inlineStr">
-        <is>
-          <t>Post-structuralisme</t>
-        </is>
-      </c>
-      <c r="L131" s="48" t="inlineStr">
-        <is>
-          <t>philosophe français qui porta le « sens du monde », la communauté, le corps et le toucher.</t>
-        </is>
-      </c>
       <c r="N131" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
         </is>
       </c>
     </row>
-    <row r="132" ht="201" customHeight="1" s="49">
+    <row r="132" ht="164.25" customHeight="1" s="49">
       <c r="A132" s="54" t="n">
         <v>1940</v>
       </c>
-      <c r="B132" s="54" t="n">
+      <c r="B132" s="54" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="C132" s="54" t="inlineStr">
+        <is>
+          <t>1940 – 2021</t>
+        </is>
+      </c>
+      <c r="D132" s="55" t="inlineStr">
+        <is>
+          <t>Jean-Luc NANCY</t>
+        </is>
+      </c>
+      <c r="E132" s="62" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jean-Luc_Nancy"  title=" Wikipedia"&gt;Jean-Luc NANCY&lt;/a&gt; était un philosophe français, agrégé de philosophie, il fut professeur à l'Université de Strasbourg jusqu'à sa retraite. Sa pensée, en dialogue constant avec Heidegger, Derrida et Lacoue-Labarthe — avec lequel il collabora étroitement — porte sur le « sens du monde », la communauté, le corps et le toucher. &lt;/p&gt; &lt;p&gt; Son œuvre est marquée par le questionnement du « with » (avec), du « being-with » heideggerien. Dans &lt;em&gt;La Communauté désoeuvrée&lt;/em&gt; (1986), il développe une pensée de la communauté qui refuse toute forme d'immanentisme ou de fusion : la communauté véritable n'est pas une substance commune, mais  &lt;a href="https://www.youtube.com/watch?v=fZK6pEAPxEw"  title="jean luc Nancy par Institut Humanités "&gt;l'exposition partagée &lt;/a&gt; de la singularité de chacun. Cette réflexion, en dialogue critique avec Blanchot et Bataille, a eu un retentissement considérable dans les débats contemporains sur la politique, la communauté et l'identité. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Corpus&lt;/em&gt; (1992) et &lt;em&gt;Noli me tangere&lt;/em&gt; (2003), il explore  &lt;a href="https://www.youtube.com/watch?v=1kCExw6Wp9k"  title="jean luc Nancy par Lacan TV "&gt;la philosophie du corps &lt;/a&gt; et du toucher comme modes fondamentaux de l'être-au-monde. Son essai sur le sens — &lt;em&gt;Le Sens du monde&lt;/em&gt; (1993) — aborde la question de la possibilité du sens dans un monde déserté par les transcendances. &lt;em&gt;L'Intrus&lt;/em&gt; (2000), bref récit autobiographique sur sa transplantation cardiaque, mêle réflexion philosophique et expérience personnelle de la maladie et de l'altérité. Son œuvre, immense et diverse, témoigne d'une pensée vivante et rigoureuse toujours en dialogue avec la littérature, l'art et la politique. &lt;/p&gt;  &lt;audio controls title="Jean luc Nancy par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/11472-06.02.2011-ITEMA_20267545-2011C16153E0003-ITE_00040439_RSCE-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
+        </is>
+      </c>
+      <c r="F132" s="54" t="inlineStr">
+        <is>
+          <t>0ONnn-EL0BA</t>
+        </is>
+      </c>
+      <c r="G132" s="56" t="inlineStr">
+        <is>
+          <t>"Jean-Luc Nancy, philosophe à l'intelligence sensible" par France Culture</t>
+        </is>
+      </c>
+      <c r="H132" s="62" t="inlineStr">
+        <is>
+          <t>https://www.laphilo.fr/pho/jlnancy-mini.webp</t>
+        </is>
+      </c>
+      <c r="J132" s="48" t="inlineStr">
+        <is>
+          <t>metaphysique ; politique</t>
+        </is>
+      </c>
+      <c r="K132" s="48" t="inlineStr">
+        <is>
+          <t>Post-structuralisme</t>
+        </is>
+      </c>
+      <c r="L132" s="48" t="inlineStr">
+        <is>
+          <t>philosophe français qui porta le « sens du monde », la communauté, le corps et le toucher.</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="201" customHeight="1" s="49">
+      <c r="A133" s="54" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B133" s="54" t="n">
         <v>2007</v>
       </c>
-      <c r="C132" s="54" t="inlineStr">
+      <c r="C133" s="54" t="inlineStr">
         <is>
           <t>1940 – 2007</t>
         </is>
       </c>
-      <c r="D132" s="55" t="inlineStr">
+      <c r="D133" s="55" t="inlineStr">
         <is>
           <t>Philippe LACOUE-LABARTHE</t>
         </is>
       </c>
-      <c r="E132" s="62" t="inlineStr">
+      <c r="E133" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Philippe_Lacoue-Labarthe"  title=" Wikipedia"&gt;Philippe LACOUE-LABARTHE&lt;/a&gt; était un philosophe, critique littéraire, traducteur et théoricien français né à Tours et connu pour ses travaux sur la mimésis, le romantisme allemand, Hölderlin, Heidegger, Derrida et la relation entre esthétique et politique. Il a aussi beaucoup compté dans le milieu intellectuel de Strasbourg, où il a enseigné longtemps et travaillé avec Jean-Luc Nancy. &lt;/p&gt; &lt;p&gt; Son  &lt;a href="https://maitron.fr/lacoue-labarthe-philippe/"  title=" lacoue-labarthe par le maitron"&gt;œuvre interroge &lt;/a&gt; la façon dont l’art, la philosophie et la politique s’entrecroisent, notamment à travers la notion de mimésis et la critique de l’“esthétisation du politique”. Il a aussi travaillé sur le romantisme allemand et sur la réception de Hölderlin, qu’il considérait comme une figure majeure. &lt;/p&gt; &lt;p&gt; Parmi les livres souvent cités, on trouve Le Titre de la lettre avec Jean-Luc Nancy, L’Absolu littéraire, L’Imitation des modernes, La Fiction du politique et Heidegger, la politique du poème. Il a également traduit plusieurs auteurs allemands majeurs, dont Heidegger, Hölderlin, Nietzsche, Benjamin et Celan. &lt;/p&gt; &lt;p&gt; Sa pensée tourne autour de trois idées principales : La représentation n’est jamais transparente : ce que nous montrons, racontons ou jouons n’est jamais la réalité elle-même, mais une forme, un masque, une imitation. La littérature et le théâtre sont essentiels pour comprendre la philosophie, parce qu’ils révèlent ce que les concepts cachent ou simplifient.popups. Le lien entre esthétique et politique est dangereux : il a beaucoup réfléchi à la manière dont l’art, les mythes et les images peuvent servir le politique, y compris dans des formes fascisantes. &lt;/p&gt; 
  &lt;audio controls title="les versions de philippe lacoue labarthe par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/16409-16.03.2007-ITEMA_20062386-2007C6409S0011-MEM_000036772_RF-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
         </is>
       </c>
-      <c r="F132" s="54" t="inlineStr">
+      <c r="F133" s="54" t="inlineStr">
         <is>
           <t>CI6zYPSwsoY</t>
         </is>
       </c>
-      <c r="G132" s="56" t="inlineStr">
+      <c r="G133" s="56" t="inlineStr">
         <is>
           <t>voyage a tubingen par capuseen</t>
         </is>
       </c>
-      <c r="H132" s="62" t="inlineStr">
+      <c r="H133" s="62" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/pllabarthe-mini.webp</t>
         </is>
       </c>
-      <c r="J132" s="48" t="inlineStr">
+      <c r="J133" s="48" t="inlineStr">
         <is>
           <t>politique ; epistemologie</t>
         </is>
       </c>
-      <c r="K132" s="48" t="inlineStr">
+      <c r="K133" s="48" t="inlineStr">
         <is>
           <t>Déconstructionnisme</t>
         </is>
       </c>
-      <c r="L132" s="85" t="inlineStr">
+      <c r="L133" s="85" t="inlineStr">
         <is>
           <t xml:space="preserve"> philosophe et théoricien français connu pour ses travaux sur la mimésis et le romantisme allemand.</t>
         </is>
       </c>
-      <c r="N132" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="209.25" customHeight="1" s="49">
-      <c r="A133" s="57" t="n">
+      <c r="N133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="209.25" customHeight="1" s="49">
+      <c r="A134" s="57" t="n">
         <v>1941</v>
       </c>
-      <c r="B133" s="57" t="inlineStr">
+      <c r="B134" s="57" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="C133" s="57" t="inlineStr">
+      <c r="C134" s="57" t="inlineStr">
         <is>
           <t>1941 – 2019</t>
         </is>
       </c>
-      <c r="D133" s="58" t="inlineStr">
+      <c r="D134" s="58" t="inlineStr">
         <is>
           <t>François DELAPORTE</t>
         </is>
       </c>
-      <c r="E133" s="59" t="inlineStr">
+      <c r="E134" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Fran%C3%A7ois_Delaporte"  title=" Wikipedia"&gt;François DELAPORTE&lt;/a&gt; était un philosophe français spécialiste d'histoire et de philosophie des sciences médicales et biologiques, connu notamment pour ses travaux sur l'histoire des maladies et la philosophie de Georges Canguilhem. Professeur à l'Université de Picardie, il fut l'un des continuateurs de la tradition canguilhémienne d'histoire et philosophie des sciences en France, appliquant cette approche à l'histoire de la médecine et de la biologie. &lt;/p&gt; &lt;p&gt; Son œuvre la plus importante, &lt;em&gt;   &lt;a href="https://www.persee.fr/doc/bec_0373-6237_1993_num_151_2_450700_t1_0415_0000_001"  title=" le savoir sur la maladie par persée"&gt;Le Savoir de la maladie. &lt;/a&gt; Essai sur le choléra de 1832 à Paris&lt;/em&gt; (1990), est une analyse philosophique de l'épidémie de choléra qui ravagea Paris en 1832. Suivant la méthode de Canguilhem et Foucault, il montre comment la compréhension d'une maladie est toujours insérée dans un réseau de savoirs, de pratiques et de pouvoirs qui configurent sa signification médicale et sociale. Cette étude est un modèle du genre pour l'articulation entre histoire des sciences et analyse philosophique. &lt;/p&gt; &lt;p&gt; Il contribua également à faire connaître la pensée de Canguilhem, notamment à travers des études sur &lt;em&gt;Le Normal et le Pathologique&lt;/em&gt; et sur la philosophie biologique canguilhémienne. Ses travaux sur l'histoire des figures du visage, réunis dans &lt;em&gt;Figures de la médecine&lt;/em&gt; (2009), constituent une autre contribution originale à l'intersection de l'histoire de l'art médical et de la philosophie du corps. Delaporte incarne une tradition française de philosophie de la médecine d'une grande rigueur et d'une réelle originalité. &lt;/p&gt;   &lt;audio controls title="François Laporte le vie monastique, pensée en mouvement  par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/11983-19.12.2013-ITEMA_20563752-2013C18137S0353-25.m4a" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
         </is>
       </c>
-      <c r="F133" s="57" t="inlineStr">
+      <c r="F134" s="57" t="inlineStr">
         <is>
           <t>Y3FnglRhPxs</t>
         </is>
       </c>
-      <c r="G133" s="59" t="inlineStr">
+      <c r="G134" s="59" t="inlineStr">
         <is>
           <t>"François DELAPORTE 2014" par Colin Guillaume</t>
         </is>
       </c>
-      <c r="H133" s="65" t="inlineStr">
+      <c r="H134" s="65" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/fdelaporte-mini.webp</t>
         </is>
       </c>
-      <c r="J133" s="48" t="inlineStr">
+      <c r="J134" s="48" t="inlineStr">
         <is>
           <t>epistemologie</t>
         </is>
       </c>
-      <c r="K133" s="48" t="inlineStr">
+      <c r="K134" s="48" t="inlineStr">
         <is>
           <t>Constructivisme</t>
         </is>
       </c>
-      <c r="L133" s="48" t="inlineStr">
+      <c r="L134" s="48" t="inlineStr">
         <is>
           <t>philosophe français spécialiste de philosophie des sciences médicales et biologiques.</t>
         </is>
       </c>
-      <c r="N133" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="218.25" customHeight="1" s="49">
-      <c r="A134" s="54" t="n">
+      <c r="N134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="218.25" customHeight="1" s="49">
+      <c r="A135" s="54" t="n">
         <v>1944</v>
       </c>
-      <c r="B134" s="54" t="inlineStr">
+      <c r="B135" s="54" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C134" s="54" t="inlineStr">
+      <c r="C135" s="54" t="inlineStr">
         <is>
           <t>1944 – 2022</t>
         </is>
       </c>
-      <c r="D134" s="55" t="inlineStr">
+      <c r="D135" s="55" t="inlineStr">
         <is>
           <t>Dominique LECOURT</t>
         </is>
       </c>
-      <c r="E134" s="63" t="inlineStr">
+      <c r="E135" s="63" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Dominique_Lecourt" title=" Wikipedia"&gt;Dominique LECOURT&lt;/a&gt; était un philosophe français connu pour ses travaux en philosophie des sciences et pour avoir prolongé, de manière originale, l’héritage de Gaston Bachelard et de Georges Canguilhem. Sa philosophie se déploie autour de la philosophie des sciences, des rapports entre savoir et pouvoir, et d’une réflexion éthique et politique sur la technoscience. &lt;/p&gt; &lt;p&gt; Disciple de Bachelard, il défend un "rationalisme appliqué" : la raison scientifique n’est pas une abstraction pure, mais une activité qui se confronte à des obstacles, des erreurs, des idéologies, et qui progresse en les surmontant. Dans cet esprit, il insiste sur le rôle des   &lt;a href="https://www.youtube.com/watch?v=YyntmVUC1wE"  title=" D Lecourt par booksmag"&gt;"obstacles épistémologiques" &lt;/a&gt;  qui déroutent la recherche et qu’il faut analyser pour comprendre les progrès de la science. Il montre aussi que l’imagination n’est pas l’ennemie de la science : elle est indispensable à l’invention scientifique autant qu’à la rigueur des démonstrations. &lt;/p&gt; &lt;p&gt; Il cherche à contrer à la fois  l’"arrogance du scientisme"  et la technophobie ou le catastrophisme qui voient dans la technique uniquement une menace. Pour lui, la philosophie des sciences doit donner les moyens de penser la puissance des technosciences sans la sacraliser ni la diaboliser. Cela implique un dialogue étroit avec les scientifiques, mais aussi avec les juristes, médecins, sociologues, responsables politiques, pour éclairer les choix collectifs. &lt;/p&gt; &lt;p&gt; Il développe une conception de la liberté qui refuse aussi bien l’individualisme égoïste que le "moralisme libertaire". La liberté, pour lui, se joue dans le rapport aux savoirs et aux techniques : il s’agit d’en faire des instruments d’émancipation plutôt que de domination.&lt;/p&gt; &lt;p&gt; Parmi ses nombreux livres (plus d’une trentaine), on peut citer : -"Lyssenko, histoire réelle d’une "science prolétarienne" : analyse de la manipulation politique de la biologie en URSS. "L’Amérique entre la Bible et Darwin" : sur les tensions entre science et religion aux États‑Unis. "Contre la peur" : proposition d’une éthique de la recherche qui affirme la valeur de l’esprit critique face aux discours alarmistes. &lt;a href="https://www.youtube.com/watch?v=3e2K5Ogywl4"  title=" De quoi le transhumanisme est-il le nom ? par Editions M-Editer"&gt;"Humain post‑humain" &lt;/a&gt;  : réflexion sur les promesses et les dangers du transhumanisme. &lt;/p&gt;   &lt;audio controls title="L'age de la peur par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10075-03.03.2010-ITEMA_20218172-2010C6608S0062-NET_E99ABA70-9EA1-4399-B0F4-9460EA040C60-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;  </t>
         </is>
       </c>
-      <c r="F134" s="54" t="inlineStr">
+      <c r="F135" s="54" t="inlineStr">
         <is>
           <t>YyntmVUC1wE</t>
         </is>
       </c>
-      <c r="G134" s="56" t="inlineStr">
+      <c r="G135" s="56" t="inlineStr">
         <is>
           <t>"D Lecourt" par Booksmag</t>
         </is>
       </c>
-      <c r="H134" s="62" t="inlineStr">
+      <c r="H135" s="62" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/lecourt-mini.webp</t>
         </is>
       </c>
-      <c r="J134" s="48" t="inlineStr">
+      <c r="J135" s="48" t="inlineStr">
         <is>
           <t>epistemologie</t>
         </is>
       </c>
-      <c r="K134" s="48" t="inlineStr">
+      <c r="K135" s="48" t="inlineStr">
         <is>
           <t>Marxisme ; Constructivisme</t>
         </is>
       </c>
-      <c r="L134" s="48" t="inlineStr">
+      <c r="L135" s="48" t="inlineStr">
         <is>
           <t>philosophe français connu pour ses travaux en philosophie des sciences.</t>
         </is>
       </c>
-      <c r="N134" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="157.5" customHeight="1" s="49">
-      <c r="A135" s="57" t="n">
+      <c r="N135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="157.5" customHeight="1" s="49">
+      <c r="A136" s="57" t="n">
         <v>1945</v>
       </c>
-      <c r="B135" s="57" t="inlineStr">
+      <c r="B136" s="57" t="inlineStr">
         <is>
           <t>2006</t>
         </is>
       </c>
-      <c r="C135" s="57" t="inlineStr">
+      <c r="C136" s="57" t="inlineStr">
         <is>
           <t>1945 – 2006</t>
         </is>
       </c>
-      <c r="D135" s="58" t="inlineStr">
+      <c r="D136" s="58" t="inlineStr">
         <is>
           <t>Jean-Michel BERTHELOT</t>
         </is>
       </c>
-      <c r="E135" s="65" t="inlineStr">
+      <c r="E136" s="65" t="inlineStr">
         <is>
           <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Jean-Michel_Berthelot"  title=" Wikipedia"&gt;Jean-Michel BERTHELOT&lt;/a&gt; était un philosophe et sociologue français spécialiste d'épistémologie des sciences sociales. Professeur à l'Université de Paris IV-Sorbonne et à l'Université du Québec à Montréal, il contribua de manière décisive à la réflexion philosophique sur les fondements et les méthodes des sciences humaines et sociales. Son œuvre joint la rigueur épistémologique à une large culture philosophique et sociologique. &lt;/p&gt; &lt;p&gt; Son ouvrage principal, &lt;em&gt; &lt;a href="https://www.persee.fr/doc/sotra_0038-0296_1992_num_34_3_2605_t1_0388_0000_3"  title="l’intelligence du social par persée "&gt; L'Intelligence du social&lt;/a&gt; &lt;/em&gt; (1990), est une analyse approfondie des schèmes d'intelligibilité que les sciences sociales utilisent pour rendre compte de la réalité sociale : le schème causal, le schème fonctionnel, le schème structural, le schème herméneutique et d'autres modes d'explication. Berthelot montre que chaque paradigme sociologique privilégie un mode d'intelligibilité particulier, ce qui permet de comprendre à la fois leurs apports spécifiques et leurs limites. Ce livre constitue l'une des contributions les plus claires et les plus systématiques à la philosophie des sciences sociales en langue française. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Epistémologie des sciences sociales&lt;/em&gt; (2001, ouvrage collectif qu'il dirigea), il offrit un panorama complet des questions épistémologiques fondamentales que posent les sciences humaines et sociales : la causalité, la compréhension, la mesure, la modélisation, la réflexivité et les rapports entre science et valeurs. Ses travaux contribuèrent à établir l'épistémologie des sciences sociales comme une discipline à part entière dans le paysage universitaire français, en dialogue constant avec la philosophie des sciences anglophones et continentale. &lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F135" s="57" t="inlineStr">
+      <c r="F136" s="57" t="inlineStr">
         <is>
           <t>032-iGqk37A</t>
         </is>
       </c>
-      <c r="G135" s="59" t="inlineStr">
+      <c r="G136" s="59" t="inlineStr">
         <is>
           <t>"JM BERTHELOT" par SFCR</t>
         </is>
       </c>
-      <c r="H135" s="65" t="inlineStr">
+      <c r="H136" s="65" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/jmberthelot-mini.webp</t>
         </is>
       </c>
-      <c r="J135" s="48" t="inlineStr">
+      <c r="J136" s="48" t="inlineStr">
         <is>
           <t>epistemologie</t>
         </is>
       </c>
-      <c r="K135" s="48" t="inlineStr">
+      <c r="K136" s="48" t="inlineStr">
         <is>
           <t>Constructivisme</t>
         </is>
       </c>
-      <c r="L135" s="48" t="inlineStr">
+      <c r="L136" s="48" t="inlineStr">
         <is>
           <t>philosophe et sociologue français spécialiste d'épistémologie des sciences sociales.</t>
         </is>
       </c>
-      <c r="N135" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" ht="166.5" customHeight="1" s="49">
-      <c r="A136" s="54" t="n">
+      <c r="N136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="166.5" customHeight="1" s="49">
+      <c r="A137" s="54" t="n">
         <v>1946</v>
       </c>
-      <c r="B136" s="54" t="inlineStr">
+      <c r="B137" s="54" t="inlineStr">
         <is>
           <t>2010</t>
         </is>
       </c>
-      <c r="C136" s="54" t="inlineStr">
+      <c r="C137" s="54" t="inlineStr">
         <is>
           <t>1946 – 2010</t>
         </is>
       </c>
-      <c r="D136" s="55" t="inlineStr">
+      <c r="D137" s="55" t="inlineStr">
         <is>
           <t>Daniel BENSAÏD</t>
         </is>
       </c>
-      <c r="E136" s="62" t="inlineStr">
+      <c r="E137" s="62" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Daniel_Bensa%C3%AFd"  title=" Wikipedia"&gt;Daniel BENSAÏD&lt;/a&gt; était un philosophe français marxiste, l'un des intellectuels les plus importants de la gauche radicale française de son époque. Né à Paris dans une famille juive d'origine algérienne, il fut l'un des leaders de la révolte étudiante de mai 1968 à Paris-Nanterre aux côtés de Daniel Cohn-Bendit. Professeur de philosophie à l'Université Paris VIII-Saint-Denis, il fut membre dirigeant de la Ligue communiste révolutionnaire (LCR) et de son successeur le Nouveau Parti Anticapitaliste (NPA). &lt;/p&gt; &lt;p&gt; Sa pensée philosophique chercha à renouveler le marxisme en le débarrassant des &lt;a href="https://www.youtube.com/watch?v=uxBvxfRI2CE"  title="la privatisation du monde par bibou11slalala "&gt; simplifications téléologiques &lt;/a&gt; et en l'ouvrant à des problématiques nouvelles. Dans &lt;em&gt;Marx l'intempestif&lt;/em&gt; (1995), il défend un Marx débarrassé du déterminisme historique et de la philosophie du progrès, un Marx « intempestif » qui pense la politique comme art du possible et de l'impossible, en dialogue avec Blaise Pascal et Walter Benjamin. Ce livre renouvela profondément la  &lt;a href="https://www.youtube.com/watch?v=is8Ya038-Q4"  title="l’héritage de Marx par socialtram "&gt; lecture de Marx &lt;/a&gt; dans la gauche française. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Le Pari mélancolique&lt;/em&gt; (1997) et &lt;em&gt;Résistances&lt;/em&gt; (2001), il développe une philosophie de l'engagement politique nourrie par la mélancolie des défaites mais portée par une fidélité irréductible à l'émancipation. Sa réflexion sur les rapports entre philosophie et politique, entre utopie et stratégie, constitue l'une des contributions les plus originales à la pensée marxiste contemporaine. Polémiste redoutable et pédagogue exigeant, il laissa une empreinte profonde sur plusieurs générations de militants et d'intellectuels de gauche. &lt;/p&gt;  &lt;audio controls title="Daniel Bensaid  par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10075-11.12.2006-ITEMA_20049670-2006C6608S0221-MEM_000033324_RF-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F136" s="54" t="inlineStr">
+      <c r="F137" s="54" t="inlineStr">
         <is>
           <t>xFJLPfAwApo</t>
         </is>
       </c>
-      <c r="G136" s="56" t="inlineStr">
+      <c r="G137" s="56" t="inlineStr">
         <is>
           <t>"Daniel Bensaïd sur l'idée du communisme" par Videos Politiques</t>
         </is>
       </c>
-      <c r="H136" s="62" t="inlineStr">
+      <c r="H137" s="62" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/bensaid-mini.webp</t>
         </is>
       </c>
-      <c r="J136" s="48" t="inlineStr">
+      <c r="J137" s="48" t="inlineStr">
         <is>
           <t>politique</t>
         </is>
       </c>
-      <c r="K136" s="48" t="inlineStr">
+      <c r="K137" s="48" t="inlineStr">
         <is>
           <t>Marxisme</t>
         </is>
       </c>
-      <c r="L136" s="48" t="inlineStr">
+      <c r="L137" s="48" t="inlineStr">
         <is>
           <t>philosophe français marxiste, intellectuel important de la gauche radicale française.</t>
         </is>
       </c>
-      <c r="M136" t="inlineStr">
+      <c r="M137" t="inlineStr">
         <is>
           <t xml:space="preserve">juive</t>
         </is>
       </c>
-      <c r="N136" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="210" customHeight="1" s="49">
-      <c r="A137" s="57" t="n">
+      <c r="N137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="210" customHeight="1" s="49">
+      <c r="A138" s="57" t="n">
         <v>1947</v>
       </c>
-      <c r="B137" s="57" t="inlineStr">
+      <c r="B138" s="57" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C137" s="57" t="inlineStr">
+      <c r="C138" s="57" t="inlineStr">
         <is>
           <t>1947 - 2022</t>
         </is>
       </c>
-      <c r="D137" s="58" t="inlineStr">
+      <c r="D138" s="58" t="inlineStr">
         <is>
           <t>Bruno LATOUR</t>
         </is>
       </c>
-      <c r="E137" s="59" t="inlineStr">
+      <c r="E138" s="59" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bruno_Latour"  title=" Wikipedia"&gt;Bruno LATOUR&lt;/a&gt;  est un sociologue, anthropologue et philosophe français connu pour ses travaux sur la sociologie des sciences, la philosophie des sciences et l'anthropologie des modernes.&lt;/p&gt; &lt;p&gt; L'un des concepts clés développés par Latour est celui de l'acteur-réseau, également connu sous le nom de &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A9orie_de_l%27acteur-r%C3%A9seau"  title="Théorie de l'acteur-réseau par Wikipedia "&gt; théorie de l'acteur-réseau (ANT)&lt;/a&gt;. Selon cette approche, les acteurs humains et non humains sont considérés comme des "actants" qui agissent en collaboration pour produire des réalités sociales complexes. L'ANT remet en question la distinction traditionnelle entre les sujets humains et les objets inanimés, soulignant plutôt les relations et les interactions entre eux. &lt;/p&gt; &lt;p&gt; Il s'est  intéressé aux enjeux environnementaux et a contribué au développement de l'écologie politique. Il a souligné l'importance de prendre en compte les dimensions politiques et sociales dans la compréhension des questions écologiques et climatiques. Son livre &lt;a href="http://www.bruno-latour.fr/sites/default/files/uploads/TELERAMA.pdf"  title="Nous n'avons jamais été moderne par Bruno-Latour "&gt; "Nous n'avons jamais été modernes" &lt;/a&gt; (1991) remet en question la distinction entre nature et culture, mettant en lumière les façons dont les sciences et les technologies façonnent notre compréhension du monde. &lt;/p&gt; &lt;p&gt; En plus de ses travaux académiques, Bruno Latour a également participé à des &lt;a href="https://profondeurdechamps.com/2012/10/19/entretien-avec-bruno-latour-12-lart-et-la-science/"  title="L'art et la science par Profondeurdechamps "&gt; projets artistiques &lt;/a&gt; et curatoriaux. Il a collaboré avec des artistes contemporains et a contribué à des expositions d'art qui explorent les thèmes de la science, de la technologie et de l'environnement.&lt;/p&gt; &lt;audio controls title="Introduction à la pensée de Bruno LATOUR par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/22676-06.05.2022-ITEMA_23017705-2022F45096S0126-22.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; </t>
         </is>
       </c>
-      <c r="F137" s="57" t="inlineStr">
+      <c r="F138" s="57" t="inlineStr">
         <is>
           <t>BqM-sk_ZLeU</t>
         </is>
       </c>
-      <c r="G137" s="65" t="inlineStr">
+      <c r="G138" s="65" t="inlineStr">
         <is>
           <t>"Ce virus est là pour nous préparer au nouveau régime climatique" par France Culture</t>
         </is>
       </c>
-      <c r="H137" s="65" t="inlineStr">
+      <c r="H138" s="65" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/latour-mini.webp</t>
         </is>
       </c>
-      <c r="J137" s="48" t="inlineStr">
+      <c r="J138" s="48" t="inlineStr">
         <is>
           <t>epistemologie ; politique</t>
         </is>
       </c>
-      <c r="K137" s="48" t="inlineStr">
+      <c r="K138" s="48" t="inlineStr">
         <is>
           <t>Constructivisme</t>
         </is>
       </c>
-      <c r="L137" s="48" t="inlineStr">
+      <c r="L138" s="48" t="inlineStr">
         <is>
           <t>philosophe français inscrit dans le mouvement du Nouveau Réalisme.</t>
         </is>
       </c>
-      <c r="N137" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="166.5" customHeight="1" s="49">
-      <c r="A138" s="54" t="n">
+      <c r="N138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="166.5" customHeight="1" s="49">
+      <c r="A139" s="54" t="n">
         <v>1949</v>
       </c>
-      <c r="B138" s="54" t="inlineStr">
+      <c r="B139" s="54" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
       </c>
-      <c r="C138" s="54" t="inlineStr">
+      <c r="C139" s="54" t="inlineStr">
         <is>
           <t>1949 – 2017</t>
         </is>
       </c>
-      <c r="D138" s="55" t="inlineStr">
+      <c r="D139" s="55" t="inlineStr">
         <is>
           <t>Robert DAMIEN</t>
         </is>
       </c>
-      <c r="E138" s="56" t="inlineStr">
+      <c r="E139" s="56" t="inlineStr">
         <is>
           <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Robert_Damien"  title=" Wikipedia"&gt;Robert DAMIEN&lt;/a&gt;   était un philosophe français  spécialiste de l'autorité politique et des tensions démocratiques, connu pour sa réhabilitation éthique de l'autorité comme principe d'élévation collective. Il incarna un rationalisme républicain franc et dialogique. &lt;/p&gt; &lt;p&gt; Il réfléchit aux tensions indépassables de la démocratie : décision vs connaissance, immanence vs autorité, pluralisme vs unité. L'autorité n'est pas abus ou force, mais "augmentation" (étymologiquement) : réciproque, fraternelle, légitime si elle élève sans domination, en rendant des comptes publics. Il prône un "pluralisme cohérent" (inspiré de Bachelard), un cogito relationnel et un État stratège sous souverainetés plurielles, face au déclin des absolus. &lt;/p&gt; &lt;p&gt; Joueur et &lt;a href="https://www.dailymotion.com/video/x18br7c" title="Robert Damien : de la figure de l'entraîneur à celle de Mandela par mediapart"&gt;entraîneur de rugby &lt;/a&gt; au CS Lons-le-Saunier, il intégrait le sport comme modèle philosophique du collectif et de l'autorité républicaine. Le rugby incarne pour lui une coopération interdépendante où la diversité des talents (puissants et habiles) fusionne en "Nous" : circulation du ballon prime sur l'individualisme, reliant partenaires contre adversaire. Pas de "joueurs isolés", mais des équipes où le "jeu sans ballon" (replacements, soutiens obscurs) assure continuité, révélant un "Moi nouveau" via le collectif. Dans "Activité physique et exercices spirituels" paru en 2005, le sport n'est pas idéologique mais matrice de fraternité : effort charnel révèle puissances collectives, appliquées à politique et bibliothèques (pluralité ordonnée). &lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F138" s="54" t="inlineStr">
+      <c r="F139" s="54" t="inlineStr">
         <is>
           <t>iBriZ4Lhzfg</t>
         </is>
       </c>
-      <c r="G138" s="56" t="inlineStr">
+      <c r="G139" s="56" t="inlineStr">
         <is>
           <t>"robert damien les trois qualites de l autorite" par Sylvie Formero</t>
         </is>
       </c>
-      <c r="H138" s="62" t="inlineStr">
+      <c r="H139" s="62" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/rdamien-mini.webp</t>
         </is>
       </c>
-      <c r="J138" s="48" t="inlineStr">
+      <c r="J139" s="48" t="inlineStr">
         <is>
           <t>politique ; epistemologie</t>
         </is>
       </c>
-      <c r="K138" s="48" t="inlineStr">
+      <c r="K139" s="48" t="inlineStr">
         <is>
           <t>Herméneutique</t>
         </is>
       </c>
-      <c r="L138" s="48" t="inlineStr">
+      <c r="L139" s="48" t="inlineStr">
         <is>
           <t>religieux français spécialiste de l'autorité politique &amp; des tensions démocratiques.</t>
         </is>
       </c>
-      <c r="N138" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="210.75" customHeight="1" s="49">
-      <c r="A139" s="57" t="n">
+      <c r="N139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="210.75" customHeight="1" s="49">
+      <c r="A140" s="57" t="n">
         <v>1950</v>
       </c>
-      <c r="B139" s="57" t="inlineStr">
+      <c r="B140" s="57" t="inlineStr">
         <is>
           <t>2022</t>
         </is>
       </c>
-      <c r="C139" s="57" t="inlineStr">
+      <c r="C140" s="57" t="inlineStr">
         <is>
           <t>1950 – 2022</t>
         </is>
       </c>
-      <c r="D139" s="58" t="inlineStr">
+      <c r="D140" s="58" t="inlineStr">
         <is>
           <t>Catherine COLLIOT-THELENE</t>
         </is>
       </c>
-      <c r="E139" s="65" t="inlineStr">
+      <c r="E140" s="65" t="inlineStr">
         <is>
           <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Catherine_Colliot-Th%C3%A9l%C3%A8ne" title=" Wikipedia"&gt;Catherine COLLIOT-THELENE&lt;/a&gt; était une philosophe française  majeure de la philosophie politique contemporaine, spécialiste de Max Weber et penseuse des droits, de la démocratie et de la propriété dans un cadre cosmopolitique. Membre de l’Institut universitaire de France, elle est reconnue comme une référence internationale des études wébériennes. &lt;/p&gt; &lt;p&gt; Son travail se situe au croisement de la philosophie politique et des sciences sociales, avec trois pôles principaux :  &lt;a href="https://www.youtube.com/watch?v=krUYFtq9Jww" title="Max Weber et la violence légitime de l’état par France Culture"&gt;Max Weber, la démocratie et les droits, &lt;/a&gt;  la propriété et le cosmopolitisme.  Elle traduit et commente plusieurs textes de Weber, notamment Le Savant et le politique et Les Communautés, en montrant en détail ses concepts de rationalisation, de désenchantement et de domination. &lt;/p&gt; &lt;p&gt; À partir des années 2000, elle se concentre sur les droits subjectifs, leur articulation avec l’individualisme contemporain et la transformation des rapports entre pouvoirs politiques et économiques. Elle insiste sur la nécessité de penser la normativité (ce qui doit être) à partir d’une analyse précise des structures sociales réelles, d’où son dialogue constant avec le droit, l’histoire et la sociologie. &lt;/p&gt; &lt;p&gt; Dans "La Démocratie sans “demos”  paru en 2011, elle remet en question l’identification classique entre "peuple" et "démocratie". Elle critique la superposition entre souveraineté du peuple et souveraineté territoriale de l’État, qui conduit selon elle à des versions exclusives de la démocratie. &lt;a href="https://www.youtube.com/watch?v=ps2ixtEpgYI" title="la democratie c’est le droit de resistance par Journal l’Humanitét"&gt;Sa philosophie cherche &lt;/a&gt;  une démocratie fondée sur des droits universalisables et sur la participation de tous les sujets, plutôt que sur l’appartenance à une communauté nationale préconstituée. &lt;/p&gt; &lt;p&gt; Elle refuse la séparation entre théorie pure et monde social : pour elle, la philosophie politique doit dialoguer avec les sciences sociales pour produire une critique efficace des institutions et des inégalités. Elle a accompagné, sans posture militante classique mais avec une forte implication intellectuelle, les luttes pour les droits des femmes, des exclus et des étrangers, en cherchant à fournir des outils conceptuels pour penser l’égalité aujourd’hui. &lt;/p&gt; 
  &lt;audio controls title="Les défis juridiques de la migration : existe-t-il un droit à la libre circulation ? par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/21447-09.02.2022-ITEMA_22927630-2022C27677S0040-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
-      <c r="F139" s="57" t="inlineStr">
+      <c r="F140" s="57" t="inlineStr">
         <is>
           <t>g_YhgkqNE98</t>
         </is>
       </c>
-      <c r="G139" s="59" t="inlineStr">
+      <c r="G140" s="59" t="inlineStr">
         <is>
           <t>"La démocratie des droits : de Weber à Kant", entretien avec Catherine Colliot-Thélène" par Politika</t>
         </is>
       </c>
-      <c r="H139" s="65" t="inlineStr">
+      <c r="H140" s="65" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/thelene-mini.webp</t>
         </is>
       </c>
-      <c r="J139" s="48" t="inlineStr">
+      <c r="J140" s="48" t="inlineStr">
         <is>
           <t>politique</t>
         </is>
       </c>
-      <c r="K139" s="48" t="inlineStr">
+      <c r="K140" s="48" t="inlineStr">
         <is>
           <t>Libéralisme</t>
         </is>
       </c>
-      <c r="L139" s="48" t="inlineStr">
+      <c r="L140" s="48" t="inlineStr">
         <is>
           <t>philosophe française majeure de la philosophie politique contemporaine.</t>
         </is>
       </c>
-      <c r="M139" t="inlineStr">
+      <c r="M140" t="inlineStr">
         <is>
           <t xml:space="preserve">femme</t>
         </is>
       </c>
-      <c r="N139" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="171.75" customHeight="1" s="49">
-      <c r="A140" s="54" t="n">
+      <c r="N140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="171.75" customHeight="1" s="49">
+      <c r="A141" s="54" t="n">
         <v>1952</v>
       </c>
-      <c r="B140" s="54" t="inlineStr">
+      <c r="B141" s="54" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="C140" s="54" t="inlineStr">
+      <c r="C141" s="54" t="inlineStr">
         <is>
           <t>1952 – 2020</t>
         </is>
       </c>
-      <c r="D140" s="55" t="inlineStr">
+      <c r="D141" s="55" t="inlineStr">
         <is>
           <t xml:space="preserve">Bernard STIEGLER</t>
         </is>
       </c>
-      <c r="E140" s="56" t="inlineStr">
+      <c r="E141" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bernard_Stiegler"  title=" Wikipedia"&gt;Bernard STIEGLER&lt;/a&gt; était un philosophe français, l'une des figures les plus originales et les plus influentes de la philosophie française. Né à Villebon-sur-Yvette, son parcours intellectuel fut marqué par une expérience singulière : il prépara sa thèse en philosophie pendant les cinq années qu'il passa en prison (1978-1983), condamné pour braquages. Docteur en philosophie sous la direction de Jacques Derrida, il fut directeur du département du développement culturel du Centre Pompidou puis directeur de l'Institut de Recherche et d'Innovation (IRI). &lt;/p&gt; &lt;p&gt; Son œuvre maîtresse, la trilogie &lt;em&gt;&lt;a href="https://www.youtube.com/watch?v=nwmOFXzCJUg" title="Bernard Stiegler a propos de la technique par Adrien Payet"&gt;La Technique et le Temps&lt;/a&gt; &lt;/em&gt; (1994-2001), constitue l'une des analyses philosophiques les plus ambitieuses de la technique et de ses effets sur la temporalité humaine. S'appuyant sur Simondon, Derrida et Heidegger, il y défend la thèse que l'être humain est fondamentalement un être technique : c'est par la technique — les « rétentions tertiaires », les objets qui externalisent la mémoire — que l'humain se constitue comme tel. La technique n'est pas un simple outil mais la condition même de la temporalité humaine et de la transmission culturelle. &lt;/p&gt; &lt;p&gt; Dans ses ouvrages ultérieurs — &lt;em&gt;De la misère symbolique&lt;/em&gt; (2004), &lt;em&gt;Prendre soin&lt;/em&gt; (2008), &lt;em&gt;États de choc&lt;/em&gt; (2012) — il  &lt;a href="https://www.youtube.com/watch?v=IOei5Kb1cQI" title="Bernard Stiegler par France 24"&gt;développa une critique &lt;/a&gt;  de l'économie de l'attention et du capitalisme des plateformes numériques, montrant comment ceux-ci détruisent les « savoirs faire » et « savoirs vivre » qui constituent le tissu de l'existence humaine. Sa pensée, nourrie d'une profonde inquiétude sur les effets destructeurs des industries culturelles et numériques, propose une pharmacologie de la technique : la technique est un pharmakon, à la fois poison et remède. &lt;/p&gt;  &lt;audio controls title="Bernard Stiegler : je reflechis au rapport entre technique et le mal  par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/13915-05.11.2017-ITEMA_21460251-5.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;</t>
         </is>
       </c>
-      <c r="F140" s="54" t="inlineStr">
+      <c r="F141" s="54" t="inlineStr">
         <is>
           <t>Q10Ski-xusk</t>
         </is>
       </c>
-      <c r="G140" s="56" t="inlineStr">
+      <c r="G141" s="56" t="inlineStr">
         <is>
           <t>"Mémoire et personnalité - Bernard Stiegler" par Obserbatoire B2V des Mémoires</t>
         </is>
       </c>
-      <c r="H140" s="62" t="inlineStr">
+      <c r="H141" s="62" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/bstiegler-mini.webp</t>
         </is>
       </c>
-      <c r="J140" s="48" t="inlineStr">
+      <c r="J141" s="48" t="inlineStr">
         <is>
           <t>politique ; epistemologie</t>
         </is>
       </c>
-      <c r="K140" s="48" t="inlineStr">
+      <c r="K141" s="48" t="inlineStr">
         <is>
           <t>Post-structuralisme</t>
         </is>
       </c>
-      <c r="L140" s="48" t="inlineStr">
+      <c r="L141" s="48" t="inlineStr">
         <is>
           <t>philosophe français qui fit une analyse ambitieuse de la technique et de ses effets.</t>
         </is>
       </c>
-      <c r="N140" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="135.75" customHeight="1" s="49">
-      <c r="A141" s="57" t="n">
+      <c r="N141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="135.75" customHeight="1" s="49">
+      <c r="A142" s="57" t="n">
         <v>1959</v>
       </c>
-      <c r="B141" s="57" t="inlineStr">
+      <c r="B142" s="57" t="inlineStr">
         <is>
           <t>2014</t>
         </is>
       </c>
-      <c r="C141" s="57" t="inlineStr">
+      <c r="C142" s="57" t="inlineStr">
         <is>
           <t>1959 – 2014</t>
         </is>
       </c>
-      <c r="D141" s="58" t="inlineStr">
+      <c r="D142" s="58" t="inlineStr">
         <is>
           <t>Bernard MABILLE</t>
         </is>
       </c>
-      <c r="E141" s="65" t="inlineStr">
+      <c r="E142" s="65" t="inlineStr">
         <is>
           <t>&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Bernard_Mabille_(philosophe)"  style="color:#6A142A"  title=" Wikipedia"&gt;Bernard MABILLE&lt;/a&gt; était un philosophe français spécialiste de dialectique et de philosophie hégélienne, ainsi que de métaphysique contemporaine. Agrégé de philosophie et professeur à l'Université Paris IV-Sorbonne, il fut l'un des meilleurs connaisseurs français de Hegel et contribua de manière significative au renouvellement des études hégéliennes en France dans les dernières décennies du XXe siècle. &lt;/p&gt; &lt;p&gt; Sa thèse principale, &lt;em&gt;Hegel : l'épreuve de la contingence&lt;/em&gt; (1999), est une lecture originale de la philosophie hégélienne à la lumière de la problématique de la contingence. Contre les lectures qui réduisent Hegel à un penseur du nécessaire et du rationnel, Mabille montre que la contingence est au cœur même du système hégélien et que la dialectique est précisément la méthode qui permet de penser le passage du contingent au nécessaire sans l'éliminer. Cette relecture contribua à ouvrir la philosophie hégélienne à des problématiques contemporaines. &lt;/p&gt; &lt;p&gt; Dans ses travaux sur la métaphysique et la dialectique, Mabille s'intéressa également aux rapports entre la philosophie hégélienne et la phénoménologie française, notamment Merleau-Ponty et Henry. Son enseignement à la Sorbonne forma plusieurs générations d'étudiants à la rigueur de la pensée dialectique. Sa disparition prématurée priva la philosophie française d'un penseur rigoureux dont l'œuvre, bien que de volume limité, témoigne d'une lecture profonde et originale de l'idéalisme allemand et de ses prolongements contemporains. &lt;/p&gt;</t>
         </is>
       </c>
-      <c r="F141" s="57" t="inlineStr">
+      <c r="F142" s="57" t="inlineStr">
         <is>
           <t>2ZxXXD2lk_Q</t>
         </is>
       </c>
-      <c r="G141" s="59" t="inlineStr">
+      <c r="G142" s="59" t="inlineStr">
         <is>
           <t>Bernard MABILLE par La Compagnie des indes TV</t>
         </is>
       </c>
-      <c r="H141" s="65" t="inlineStr">
+      <c r="H142" s="65" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/bnabille-mini.webp</t>
         </is>
       </c>
-      <c r="J141" s="48" t="inlineStr">
+      <c r="J142" s="48" t="inlineStr">
         <is>
           <t>metaphysique</t>
         </is>
       </c>
-      <c r="K141" s="48" t="inlineStr">
+      <c r="K142" s="48" t="inlineStr">
         <is>
           <t>Idéalisme allemand</t>
         </is>
       </c>
-      <c r="L141" s="48" t="inlineStr">
+      <c r="L142" s="48" t="inlineStr">
         <is>
           <t>philosophe français spécialiste de dialectique et de philosophie hégélienne.</t>
         </is>
       </c>
-      <c r="N141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="176.25" customHeight="1" s="49">
-      <c r="A142" s="47" t="n">
+      <c r="N142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">occident</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="176.25" customHeight="1" s="49">
+      <c r="A143" s="47" t="n">
         <v>1964</v>
       </c>
-      <c r="B142" s="47" t="n">
+      <c r="B143" s="47" t="n">
         <v>2017</v>
       </c>
-      <c r="C142" s="47" t="inlineStr">
+      <c r="C143" s="47" t="inlineStr">
         <is>
           <t>1964 – 2017</t>
         </is>
       </c>
-      <c r="D142" s="47" t="inlineStr">
+      <c r="D143" s="47" t="inlineStr">
         <is>
           <t>Anne DUFOURMANTELLE</t>
         </is>
       </c>
-      <c r="E142" s="85" t="inlineStr">
+      <c r="E143" s="85" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Anne_Dufourmantelle"  title=" Wikipedia"&gt;Anne DUFOURMANTELLE&lt;/a&gt; était une philosophe et psychanalyste française dont l’œuvre, marquée par une grande finesse d’analyse, explore la vulnérabilité humaine, le risque, le secret et l’hospitalité. Bien qu’elle ne soit pas une théoricienne du &lt;a href="https://fr.wikipedia.org/wiki/Constructivisme_(%C3%A9pist%C3%A9mologie)"  title="Constructivisme par Wikipedia"&gt;« constructivisme »&lt;/a&gt;  au sens politique ou académique strict, sa pensée entre en résonance avec une réflexion sur la manière dont nous bâtissons notre rapport au monde et à l’autre. &lt;/p&gt; &lt;p&gt; Son concept d'&lt;a href="https://www.umc.org/fr/content/what-is-radical-hospitality"  title="Qu’est ce que l’hospitalité radicale par umc"&gt;« hospitalité radicale », &lt;/a&gt; nourri de ses travaux avec Jacques Derrida, propose d'accueillir l'inconnu sans conditions, voyant dans cette ouverture une forme de résistance à la fermeture du monde. Elle invite à une éthique de la rencontre où la vulnérabilité n'est pas un défaut, mais un espace de croissance mutuelle qui défie les normes sociales établies. &lt;/p&gt; &lt;p&gt; '&lt;a href="https://www.youtube.com/watch?v=QAlsJD3IAs0"  title="L’envers du feu par Librairie mollat"&gt;Dans des ouvrages &lt;/a&gt; comme Éloge du risque, elle explore la tension entre la sécurité et l'aventure de vivre, encourageant une liberté de penser et d'aimer qui dépasse les discours ambiants. Elle percevait la psychanalyse et la philosophie comme des outils pour « traquer » les mutations invisibles de notre époque et redonner du sens à nos vies intérieures. &lt;/p&gt; &lt;p&gt; Sa disparition brutale en 2017, alors qu'elle portait secours à des enfants en mer, a été perçue comme l'incarnation ultime de son engagement philosophique : une éthique en actes où le souci de l'autre devient une responsabilité immédiate. Son héritage intellectuel reste une source d'inspiration pour ceux qui cherchent à penser la douceur, l'enfance et la résistance dans un monde en mutation. &lt;/p&gt; 
 &lt;audio controls title="Anne Dufourmantelle par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/11189-07.11.2011-ITEMA_20320628-2011C15000E0211-ITE_00045291_RSCE-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt;
 </t>
         </is>
       </c>
-      <c r="F142" s="47" t="inlineStr">
+      <c r="F143" s="47" t="inlineStr">
         <is>
           <t>PCCcMUiurLo</t>
         </is>
       </c>
-      <c r="G142" s="48" t="inlineStr">
+      <c r="G143" s="48" t="inlineStr">
         <is>
           <t>Hommage à Anne DUFOURMANTELLE par PhiloCloud</t>
         </is>
       </c>
-      <c r="H142" s="48" t="inlineStr">
+      <c r="H143" s="48" t="inlineStr">
         <is>
           <t>https://www.laphilo.fr/pho/adufourmantelle-mini.webp</t>
         </is>
       </c>
-      <c r="J142" s="48" t="inlineStr">
+      <c r="J143" s="48" t="inlineStr">
         <is>
           <t>ethique ; esthetique</t>
         </is>
       </c>
-      <c r="K142" s="48" t="inlineStr">
+      <c r="K143" s="48" t="inlineStr">
         <is>
           <t>Phénoménologie</t>
         </is>
       </c>
-      <c r="L142" s="48" t="inlineStr">
+      <c r="L143" s="48" t="inlineStr">
         <is>
           <t>philosophe et psychanalyste française fine analyste, qui explore la vulnérabilité humaine.</t>
         </is>
       </c>
-      <c r="M142" t="inlineStr">
+      <c r="M143" t="inlineStr">
         <is>
           <t xml:space="preserve">femme</t>
         </is>
       </c>
-      <c r="N142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">occident</t>
-        </is>
-      </c>
-    </row>
-    <row r="143" ht="176.25" customHeight="1" s="49">
-      <c r="A143" s="47">
-        <v>1881</v>
-      </c>
-      <c r="B143" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1955</t>
-        </is>
-      </c>
-      <c r="C143" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1881 – 1955</t>
-        </is>
-      </c>
-      <c r="D143" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pierre TEILHARD DE CHARDIN</t>
-        </is>
-      </c>
-      <c r="E143" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pierre_Teilhard_de_Chardin" title=" Wikipedia"&gt;Pierre TEILHARD DE CHARDIN&lt;/a&gt; est un prêtre jésuite, paléontologue et philosophe français, qui a voulu réconcilier la foi chrétienne et la théorie de l’évolution. Né en Auvergne, il entre chez les jésuites et devient un spécialiste reconnu de la &lt;a href="https://fr.wikipedia.org/wiki/Pal%C3%A9ontologie" title=" Wikipedia"&gt;paléontologie&lt;/a&gt;. Brancardier pendant la Première Guerre mondiale, il passe ensuite plus de vingt ans en Chine, où il participe aux recherches sur l’&lt;a href="https://fr.wikipedia.org/wiki/Homme_de_P%C3%A9kin" title=" Wikipedia"&gt;Homme de Pékin&lt;/a&gt;, l’un des plus anciens fossiles humains connus, et prend part en 1931-1932 à la &lt;a href="https://fr.wikipedia.org/wiki/Croisi%C3%A8re_jaune" title=" Wikipedia"&gt;Croisière jaune&lt;/a&gt;, grande expédition à travers l’Asie centrale.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Phénomène humain&lt;/em&gt;, écrit dans les années 1930 et publié après sa mort, il décrit l’univers comme un grand mouvement d’évolution, de la matière à la vie, puis de la vie à la pensée. À mesure que la matière se complexifie, la conscience grandit : c’est la « loi de complexité-conscience ». Avec l’homme apparaît une nouvelle couche de la Terre, la &lt;a href="https://fr.wikipedia.org/wiki/Noosph%C3%A8re" title=" Wikipedia"&gt;noosphère&lt;/a&gt;, la sphère de la pensée, qui relie peu à peu tous les esprits.&lt;/p&gt; &lt;p&gt;Cette évolution est selon lui orientée vers un point de convergence final, le &lt;a href="https://fr.wikipedia.org/wiki/Point_Om%C3%A9ga" title=" Wikipedia"&gt;point Oméga&lt;/a&gt;, qu’il identifie au Christ cosmique, où l’humanité s’unira sans perdre la personnalité de chacun. Son autre grand texte, &lt;em&gt;Le Milieu divin&lt;/em&gt;, médite sur la présence de Dieu dans toutes les activités humaines. Ses idées inquiètent Rome, qui lui interdit de publier ses écrits philosophiques et l’éloigne de France. Il meurt à New York en 1955. Publiée après sa mort, son œuvre connaît un succès mondial, et l’on voit parfois dans la noosphère une anticipation d’Internet.&lt;/p&gt;</t>
-        </is>
-      </c>
-      <c r="H143" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/teilhard-mini.webp</t>
-        </is>
-      </c>
-      <c r="J143" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">metaphysique ; spiritualite</t>
-        </is>
-      </c>
-      <c r="K143" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Spiritualisme ; Panenthéisme</t>
-        </is>
-      </c>
-      <c r="L143" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">jésuite et paléontologue français, penseur d’une évolution cosmique orientée vers la conscience et l’esprit.</t>
-        </is>
-      </c>
       <c r="N143" t="inlineStr">
         <is>
           <t xml:space="preserve">occident</t>
         </is>
-      </c>
-      <c r="O143">
-        <v>2</v>
       </c>
     </row>
     <row r="144" ht="176.25" customHeight="1" s="49">
       <c r="A144" s="47">
-        <v>1868</v>
+        <v>1881</v>
       </c>
       <c r="B144" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1952</t>
+          <t xml:space="preserve">1955</t>
         </is>
       </c>
       <c r="C144" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1868 – 1952</t>
+          <t xml:space="preserve">1881 – 1955</t>
         </is>
       </c>
       <c r="D144" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Charles MAURRAS</t>
+          <t xml:space="preserve">Pierre TEILHARD DE CHARDIN</t>
         </is>
       </c>
       <c r="E144" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Charles_Maurras" title=" Wikipedia"&gt;Charles MAURRAS&lt;/a&gt; est un écrivain, journaliste et théoricien politique français, le maître à penser de l’&lt;a href="https://fr.wikipedia.org/wiki/Action_fran%C3%A7aise" title=" Wikipedia"&gt;Action française&lt;/a&gt;. Né en 1868 à Martigues, en Provence, il devient sourd vers quatorze ans, perd la foi, et monte à Paris, où il se fait connaître comme critique littéraire et poète, défenseur d’un classicisme inspiré de la Grèce contre le romantisme, qu’il juge source de désordre. L’affaire Dreyfus le jette dans la politique : en 1898, il justifie le faux du colonel Henry au nom de l’intérêt de l’armée et de l’État.&lt;/p&gt; &lt;p&gt;Avec son &lt;em&gt;Enquête sur la monarchie&lt;/em&gt; (1900), il convertit l’Action française à la royauté. Sa doctrine, le « nationalisme intégral », place la nation au-dessus de tout : seule une monarchie héréditaire, antiparlementaire et décentralisée pourrait garantir l’ordre et la durée que la République, gouvernement des partis et de l’opinion, détruirait. Agnostique, il défend pourtant l’Église catholique comme une force d’ordre. Il appelle sa méthode l’« empirisme organisateur » : tirer de l’histoire les lois du bon gouvernement. Il dénonce les « quatre États confédérés » qui, selon lui, rongent la France : les juifs, les protestants, les francs-maçons et les « métèques ». Cet antisémitisme d’État est au cœur de sa pensée.&lt;/p&gt; &lt;p&gt;Son quotidien, &lt;em&gt;L’Action française&lt;/em&gt;, exerce une influence considérable sur la droite et sur une partie de la jeunesse intellectuelle, malgré la condamnation du mouvement par le pape Pie XI en 1926. Maurras entre à l’Académie française en 1938. Hostile à l’Allemagne, il soutient pourtant en 1940 le maréchal Pétain, dont l’arrivée au pouvoir est pour lui une « divine surprise ». Condamné en 1945 à la réclusion à perpétuité et à la dégradation nationale pour intelligence avec l’ennemi, il s’écrie : « C’est la revanche de Dreyfus ! » Gracié pour raison de santé, il meurt en 1952. Sa pensée a durablement marqué l’extrême droite française.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pierre_Teilhard_de_Chardin" title=" Wikipedia"&gt;Pierre TEILHARD DE CHARDIN&lt;/a&gt; est un prêtre jésuite, paléontologue et philosophe français, qui a voulu réconcilier la foi chrétienne et la théorie de l’évolution. Né en Auvergne, il entre chez les jésuites et devient un spécialiste reconnu de la &lt;a href="https://fr.wikipedia.org/wiki/Pal%C3%A9ontologie" title=" Wikipedia"&gt;paléontologie&lt;/a&gt;. Brancardier pendant la Première Guerre mondiale, il passe ensuite plus de vingt ans en Chine, où il participe aux recherches sur l’&lt;a href="https://fr.wikipedia.org/wiki/Homme_de_P%C3%A9kin" title=" Wikipedia"&gt;Homme de Pékin&lt;/a&gt;, l’un des plus anciens fossiles humains connus, et prend part en 1931-1932 à la &lt;a href="https://fr.wikipedia.org/wiki/Croisi%C3%A8re_jaune" title=" Wikipedia"&gt;Croisière jaune&lt;/a&gt;, grande expédition à travers l’Asie centrale.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Phénomène humain&lt;/em&gt;, écrit dans les années 1930 et publié après sa mort, il décrit l’univers comme un grand mouvement d’évolution, de la matière à la vie, puis de la vie à la pensée. À mesure que la matière se complexifie, la conscience grandit : c’est la « loi de complexité-conscience ». Avec l’homme apparaît une nouvelle couche de la Terre, la &lt;a href="https://fr.wikipedia.org/wiki/Noosph%C3%A8re" title=" Wikipedia"&gt;noosphère&lt;/a&gt;, la sphère de la pensée, qui relie peu à peu tous les esprits.&lt;/p&gt; &lt;p&gt;Cette évolution est selon lui orientée vers un point de convergence final, le &lt;a href="https://fr.wikipedia.org/wiki/Point_Om%C3%A9ga" title=" Wikipedia"&gt;point Oméga&lt;/a&gt;, qu’il identifie au Christ cosmique, où l’humanité s’unira sans perdre la personnalité de chacun. Son autre grand texte, &lt;em&gt;Le Milieu divin&lt;/em&gt;, médite sur la présence de Dieu dans toutes les activités humaines. Ses idées inquiètent Rome, qui lui interdit de publier ses écrits philosophiques et l’éloigne de France. Il meurt à New York en 1955. Publiée après sa mort, son œuvre connaît un succès mondial, et l’on voit parfois dans la noosphère une anticipation d’Internet.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H144" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/maurras-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/teilhard-mini.webp</t>
         </is>
       </c>
       <c r="J144" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique</t>
+          <t xml:space="preserve">metaphysique ; spiritualite</t>
         </is>
       </c>
       <c r="K144" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Maurrassisme ; Conservatisme</t>
+          <t xml:space="preserve">Spiritualisme ; Panenthéisme</t>
         </is>
       </c>
       <c r="L144" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">écrivain et théoricien politique français, chef de l’Action française et du « nationalisme intégral ».</t>
+          <t xml:space="preserve">jésuite et paléontologue français, penseur d’une évolution cosmique orientée vers la conscience et l’esprit.</t>
         </is>
       </c>
       <c r="N144" t="inlineStr">
@@ -9567,50 +9572,52 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
-      <c r="O144"/>
+      <c r="O144">
+        <v>2</v>
+      </c>
     </row>
     <row r="145" ht="176.25" customHeight="1" s="49">
       <c r="A145" s="47">
-        <v>1827</v>
+        <v>1868</v>
       </c>
       <c r="B145" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1907</t>
+          <t xml:space="preserve">1952</t>
         </is>
       </c>
       <c r="C145" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1827 – 1907</t>
+          <t xml:space="preserve">1868 – 1952</t>
         </is>
       </c>
       <c r="D145" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Marcellin BERTHELOT</t>
+          <t xml:space="preserve">Charles MAURRAS</t>
         </is>
       </c>
       <c r="E145" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Marcellin_Berthelot" title=" Wikipedia"&gt;Marcellin BERTHELOT&lt;/a&gt; est un chimiste, historien des sciences et homme politique français, l’une des figures les plus représentatives du &lt;a href="https://fr.wikipedia.org/wiki/Scientisme" title=" Wikipedia"&gt;scientisme&lt;/a&gt;. Né à Paris en 1827, fils d’un médecin, il devient l’un des fondateurs de la chimie organique de synthèse : il montre qu’on peut fabriquer en laboratoire, à partir des éléments, des corps jusque-là produits seulement par les êtres vivants, comme l’acétylène, le méthane ou l’alcool. Il en tire une leçon philosophique : il n’existe pas de « force vitale » mystérieuse, la vie obéit aux mêmes lois que la matière.&lt;/p&gt; &lt;p&gt;Pour Berthelot, la science expérimentale est la seule voie vers la vérité, et elle doit aussi fonder la morale et la politique. « Le monde est aujourd’hui sans mystère », écrit-il en 1885 : ce que la science ne sait pas encore, elle le saura demain. Ami de &lt;a href="https://fr.wikipedia.org/wiki/Ernest_Renan" title=" Wikipedia"&gt;Ernest Renan&lt;/a&gt;, avec qui il partage la foi dans l’avenir de la science, il expose ses idées dans &lt;em&gt;Science et morale&lt;/em&gt; (1897). En 1895, quand le critique Ferdinand Brunetière proclame la « faillite de la science », qui n’aurait pas tenu ses promesses morales, Berthelot devient le porte-parole de la réplique républicaine et laïque.&lt;/p&gt; &lt;p&gt;Sénateur inamovible, il est ministre de l’Instruction publique (1886-1887) puis des Affaires étrangères (1895-1896), et défend une école laïque fondée sur les sciences. Professeur au Collège de France, secrétaire perpétuel de l’Académie des sciences, il s’oppose aussi à la théorie atomique, qu’il juge trop hypothétique. Il meurt en 1907 le même jour que sa femme, et tous deux sont inhumés au Panthéon.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Charles_Maurras" title=" Wikipedia"&gt;Charles MAURRAS&lt;/a&gt; est un écrivain, journaliste et théoricien politique français, le maître à penser de l’&lt;a href="https://fr.wikipedia.org/wiki/Action_fran%C3%A7aise" title=" Wikipedia"&gt;Action française&lt;/a&gt;. Né en 1868 à Martigues, en Provence, il devient sourd vers quatorze ans, perd la foi, et monte à Paris, où il se fait connaître comme critique littéraire et poète, défenseur d’un classicisme inspiré de la Grèce contre le romantisme, qu’il juge source de désordre. L’affaire Dreyfus le jette dans la politique : en 1898, il justifie le faux du colonel Henry au nom de l’intérêt de l’armée et de l’État.&lt;/p&gt; &lt;p&gt;Avec son &lt;em&gt;Enquête sur la monarchie&lt;/em&gt; (1900), il convertit l’Action française à la royauté. Sa doctrine, le « nationalisme intégral », place la nation au-dessus de tout : seule une monarchie héréditaire, antiparlementaire et décentralisée pourrait garantir l’ordre et la durée que la République, gouvernement des partis et de l’opinion, détruirait. Agnostique, il défend pourtant l’Église catholique comme une force d’ordre. Il appelle sa méthode l’« empirisme organisateur » : tirer de l’histoire les lois du bon gouvernement. Il dénonce les « quatre États confédérés » qui, selon lui, rongent la France : les juifs, les protestants, les francs-maçons et les « métèques ». Cet antisémitisme d’État est au cœur de sa pensée.&lt;/p&gt; &lt;p&gt;Son quotidien, &lt;em&gt;L’Action française&lt;/em&gt;, exerce une influence considérable sur la droite et sur une partie de la jeunesse intellectuelle, malgré la condamnation du mouvement par le pape Pie XI en 1926. Maurras entre à l’Académie française en 1938. Hostile à l’Allemagne, il soutient pourtant en 1940 le maréchal Pétain, dont l’arrivée au pouvoir est pour lui une « divine surprise ». Condamné en 1945 à la réclusion à perpétuité et à la dégradation nationale pour intelligence avec l’ennemi, il s’écrie : « C’est la revanche de Dreyfus ! » Gracié pour raison de santé, il meurt en 1952. Sa pensée a durablement marqué l’extrême droite française.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H145" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/berthelot-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/maurras-mini.webp</t>
         </is>
       </c>
       <c r="J145" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie ; politique</t>
+          <t xml:space="preserve">politique</t>
         </is>
       </c>
       <c r="K145" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scientisme ; Positivisme</t>
+          <t xml:space="preserve">Maurrassisme ; Conservatisme</t>
         </is>
       </c>
       <c r="L145" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">chimiste et homme politique français, figure emblématique du scientisme.</t>
+          <t xml:space="preserve">écrivain et théoricien politique français, chef de l’Action française et du « nationalisme intégral ».</t>
         </is>
       </c>
       <c r="N145" t="inlineStr">
@@ -9622,46 +9629,46 @@
     </row>
     <row r="146" ht="176.25" customHeight="1" s="49">
       <c r="A146" s="47">
-        <v>1861</v>
+        <v>1827</v>
       </c>
       <c r="B146" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1916</t>
+          <t xml:space="preserve">1907</t>
         </is>
       </c>
       <c r="C146" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1861 – 1916</t>
+          <t xml:space="preserve">1827 – 1907</t>
         </is>
       </c>
       <c r="D146" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pierre DUHEM</t>
+          <t xml:space="preserve">Marcellin BERTHELOT</t>
         </is>
       </c>
       <c r="E146" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pierre_Duhem" title=" Wikipedia"&gt;Pierre DUHEM&lt;/a&gt; est un physicien, philosophe et historien des sciences français. Né à Paris en 1861, brillant élève de l’École normale supérieure, il consacre ses travaux de physique à la thermodynamique. Une thèse où il critique les idées du chimiste Marcellin Berthelot est refusée ; Berthelot, très puissant, l’empêche ensuite d’obtenir un poste à Paris, et Duhem, catholique convaincu, fait sa carrière en province, à Lille, à Rennes, puis à Bordeaux.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Théorie physique, son objet, sa structure&lt;/em&gt; (1906), il soutient qu’une théorie physique n’explique pas la réalité cachée des choses, ce qui relève de la métaphysique : elle est un système de propositions mathématiques qui représente et classe le plus simplement possible les lois expérimentales. Il faut, comme disaient les astronomes grecs, « sauver les phénomènes ». Surtout, une expérience ne peut jamais réfuter une hypothèse isolée : elle met en jeu tout un ensemble de théories et d’instruments, et si la prédiction échoue, on ne sait pas laquelle des hypothèses est fausse. Il n’y a donc pas d’« expérience cruciale ». Cette idée, reprise par Quine, est connue comme la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A8se_de_Duhem-Quine" title=" Wikipedia"&gt;thèse de Duhem-Quine&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Duhem est aussi un grand historien des sciences. Dans les dix volumes du &lt;em&gt;Système du monde&lt;/em&gt;, il redécouvre la physique du Moyen Âge, celle de Jean Buridan et de Nicole Oresme, et montre que la science moderne ne naît pas d’une rupture brutale avec les siècles « obscurs », mais les prolonge. Il meurt en 1916. Son instrumentalisme et son holisme ont profondément marqué la philosophie des sciences du XXe siècle.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Marcellin_Berthelot" title=" Wikipedia"&gt;Marcellin BERTHELOT&lt;/a&gt; est un chimiste, historien des sciences et homme politique français, l’une des figures les plus représentatives du &lt;a href="https://fr.wikipedia.org/wiki/Scientisme" title=" Wikipedia"&gt;scientisme&lt;/a&gt;. Né à Paris en 1827, fils d’un médecin, il devient l’un des fondateurs de la chimie organique de synthèse : il montre qu’on peut fabriquer en laboratoire, à partir des éléments, des corps jusque-là produits seulement par les êtres vivants, comme l’acétylène, le méthane ou l’alcool. Il en tire une leçon philosophique : il n’existe pas de « force vitale » mystérieuse, la vie obéit aux mêmes lois que la matière.&lt;/p&gt; &lt;p&gt;Pour Berthelot, la science expérimentale est la seule voie vers la vérité, et elle doit aussi fonder la morale et la politique. « Le monde est aujourd’hui sans mystère », écrit-il en 1885 : ce que la science ne sait pas encore, elle le saura demain. Ami de &lt;a href="https://fr.wikipedia.org/wiki/Ernest_Renan" title=" Wikipedia"&gt;Ernest Renan&lt;/a&gt;, avec qui il partage la foi dans l’avenir de la science, il expose ses idées dans &lt;em&gt;Science et morale&lt;/em&gt; (1897). En 1895, quand le critique Ferdinand Brunetière proclame la « faillite de la science », qui n’aurait pas tenu ses promesses morales, Berthelot devient le porte-parole de la réplique républicaine et laïque.&lt;/p&gt; &lt;p&gt;Sénateur inamovible, il est ministre de l’Instruction publique (1886-1887) puis des Affaires étrangères (1895-1896), et défend une école laïque fondée sur les sciences. Professeur au Collège de France, secrétaire perpétuel de l’Académie des sciences, il s’oppose aussi à la théorie atomique, qu’il juge trop hypothétique. Il meurt en 1907 le même jour que sa femme, et tous deux sont inhumés au Panthéon.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H146" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/duhem-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/berthelot-mini.webp</t>
         </is>
       </c>
       <c r="J146" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie</t>
+          <t xml:space="preserve">epistemologie ; politique</t>
         </is>
       </c>
       <c r="K146" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instrumentalisme ; Holisme</t>
+          <t xml:space="preserve">Scientisme ; Positivisme</t>
         </is>
       </c>
       <c r="L146" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">physicien et philosophe des sciences français, pour qui une hypothèse n’est jamais testée seule.</t>
+          <t xml:space="preserve">chimiste et homme politique français, figure emblématique du scientisme.</t>
         </is>
       </c>
       <c r="N146" t="inlineStr">
@@ -9673,46 +9680,46 @@
     </row>
     <row r="147" ht="176.25" customHeight="1" s="49">
       <c r="A147" s="47">
-        <v>1854</v>
+        <v>1861</v>
       </c>
       <c r="B147" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1912</t>
+          <t xml:space="preserve">1916</t>
         </is>
       </c>
       <c r="C147" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1854 – 1912</t>
+          <t xml:space="preserve">1861 – 1916</t>
         </is>
       </c>
       <c r="D147" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Henri POINCARÉ</t>
+          <t xml:space="preserve">Pierre DUHEM</t>
         </is>
       </c>
       <c r="E147" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Henri_Poincar%C3%A9" title=" Wikipedia"&gt;Henri POINCARÉ&lt;/a&gt; est un mathématicien, physicien et philosophe des sciences français, l’un des derniers savants universels. Né à Nancy en 1854, polytechnicien et ingénieur des mines, il enseigne à la Sorbonne à partir de 1881. Il renouvelle presque toutes les branches des mathématiques : il fonde la topologie, découvre en étudiant le mouvement de trois corps célestes les comportements imprévisibles qu’on appellera « chaos », et pose en 1905, en même temps qu’Einstein, les bases mathématiques de la relativité restreinte.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Science et l’Hypothèse&lt;/em&gt; (1902), il défend le &lt;a href="https://fr.wikipedia.org/wiki/Conventionnalisme" title=" Wikipedia"&gt;conventionnalisme&lt;/a&gt; : certains principes de la science ne sont ni des vérités a priori ni des faits d’expérience, mais des conventions. Ainsi, aucune expérience ne peut dire si l’espace est euclidien ou non : nous choisissons la géométrie d’Euclide parce qu’elle est la plus commode. Ces conventions ne sont pas arbitraires, car l’expérience nous guide, mais elles ne peuvent être ni vraies ni fausses. La science ne connaît pas les choses elles-mêmes, mais les rapports entre les choses.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Valeur de la science&lt;/em&gt; (1905) et &lt;em&gt;Science et méthode&lt;/em&gt; (1908), il s’oppose aussi aux logiciens, comme Russell, qui veulent réduire les mathématiques à la logique : pour lui, le raisonnement mathématique repose sur une intuition. Il décrit le rôle de l’inconscient dans la découverte, à partir de ses propres illuminations soudaines, comme celle qui lui vint en montant dans un omnibus. Élu à l’Académie française en 1908, il meurt à Paris en 1912.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pierre_Duhem" title=" Wikipedia"&gt;Pierre DUHEM&lt;/a&gt; est un physicien, philosophe et historien des sciences français. Né à Paris en 1861, brillant élève de l’École normale supérieure, il consacre ses travaux de physique à la thermodynamique. Une thèse où il critique les idées du chimiste Marcellin Berthelot est refusée ; Berthelot, très puissant, l’empêche ensuite d’obtenir un poste à Paris, et Duhem, catholique convaincu, fait sa carrière en province, à Lille, à Rennes, puis à Bordeaux.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Théorie physique, son objet, sa structure&lt;/em&gt; (1906), il soutient qu’une théorie physique n’explique pas la réalité cachée des choses, ce qui relève de la métaphysique : elle est un système de propositions mathématiques qui représente et classe le plus simplement possible les lois expérimentales. Il faut, comme disaient les astronomes grecs, « sauver les phénomènes ». Surtout, une expérience ne peut jamais réfuter une hypothèse isolée : elle met en jeu tout un ensemble de théories et d’instruments, et si la prédiction échoue, on ne sait pas laquelle des hypothèses est fausse. Il n’y a donc pas d’« expérience cruciale ». Cette idée, reprise par Quine, est connue comme la &lt;a href="https://fr.wikipedia.org/wiki/Th%C3%A8se_de_Duhem-Quine" title=" Wikipedia"&gt;thèse de Duhem-Quine&lt;/a&gt;.&lt;/p&gt; &lt;p&gt;Duhem est aussi un grand historien des sciences. Dans les dix volumes du &lt;em&gt;Système du monde&lt;/em&gt;, il redécouvre la physique du Moyen Âge, celle de Jean Buridan et de Nicole Oresme, et montre que la science moderne ne naît pas d’une rupture brutale avec les siècles « obscurs », mais les prolonge. Il meurt en 1916. Son instrumentalisme et son holisme ont profondément marqué la philosophie des sciences du XXe siècle.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H147" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/poincare-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/duhem-mini.webp</t>
         </is>
       </c>
       <c r="J147" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">epistemologie ; logique</t>
+          <t xml:space="preserve">epistemologie</t>
         </is>
       </c>
       <c r="K147" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conventionnalisme</t>
+          <t xml:space="preserve">Instrumentalisme ; Holisme</t>
         </is>
       </c>
       <c r="L147" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">mathématicien et physicien français, philosophe des sciences et fondateur du conventionnalisme.</t>
+          <t xml:space="preserve">physicien et philosophe des sciences français, pour qui une hypothèse n’est jamais testée seule.</t>
         </is>
       </c>
       <c r="N147" t="inlineStr">
@@ -9720,52 +9727,50 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
-      <c r="O147">
-        <v>2</v>
-      </c>
+      <c r="O147"/>
     </row>
     <row r="148" ht="176.25" customHeight="1" s="49">
       <c r="A148" s="47">
-        <v>1866</v>
+        <v>1854</v>
       </c>
       <c r="B148" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1947</t>
+          <t xml:space="preserve">1912</t>
         </is>
       </c>
       <c r="C148" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1866 – 1947</t>
+          <t xml:space="preserve">1854 – 1912</t>
         </is>
       </c>
       <c r="D148" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Léon ROBIN</t>
+          <t xml:space="preserve">Henri POINCARÉ</t>
         </is>
       </c>
       <c r="E148" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/L%C3%A9on_Robin" title=" Wikipedia"&gt;Léon ROBIN&lt;/a&gt; est un philosophe et historien français de la philosophie, l’un des grands spécialistes de la pensée grecque. Né à Nantes en 1866, fils de marchand, il est reçu à l’agrégation de philosophie en 1891 et enseigne longtemps dans les lycées, à Compiègne, Vendôme et Angers. Élève et disciple d’Octave Hamelin, il publie après la mort de celui-ci son cours sur &lt;em&gt;Le Système d’Aristote&lt;/em&gt;. Il enseigne ensuite à Caen, puis à la Sorbonne de 1913 à 1937, où il occupe à partir de 1924 la chaire d’histoire de la philosophie antique.&lt;/p&gt; &lt;p&gt;Sa thèse, &lt;em&gt;La Théorie platonicienne des Idées et des nombres d’après Aristote&lt;/em&gt; (1908), s’appuie sur les témoignages d’Aristote pour reconstituer l’enseignement oral de &lt;a href="https://fr.wikipedia.org/wiki/Platon" title=" Wikipedia"&gt;Platon&lt;/a&gt; à l’Académie, où les Idées sont rattachées à des principes mathématiques, l’Un et la Dyade. Dans &lt;em&gt;La Pensée grecque et les origines de l’esprit scientifique&lt;/em&gt; (1923), il retrace la naissance de la raison grecque, des premiers physiciens d’Ionie jusqu’aux écoles hellénistiques. Il consacre aussi des livres à la morale antique, à Platon et au scepticisme de Pyrrhon, toujours appuyés sur une lecture rigoureuse des textes grecs.&lt;/p&gt; &lt;p&gt;Son œuvre la plus durable est la traduction des œuvres complètes de Platon pour la Bibliothèque de la Pléiade, qu’il dirige et dont il traduit lui-même la plus grande partie : précise et élégante, elle a fait lire Platon à des générations de lecteurs français. Il dirige aussi l’Institut international de philosophie. Il meurt à Paris en 1947. Pierre-Maxime Schuhl lui a succédé à la Sorbonne.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Henri_Poincar%C3%A9" title=" Wikipedia"&gt;Henri POINCARÉ&lt;/a&gt; est un mathématicien, physicien et philosophe des sciences français, l’un des derniers savants universels. Né à Nancy en 1854, polytechnicien et ingénieur des mines, il enseigne à la Sorbonne à partir de 1881. Il renouvelle presque toutes les branches des mathématiques : il fonde la topologie, découvre en étudiant le mouvement de trois corps célestes les comportements imprévisibles qu’on appellera « chaos », et pose en 1905, en même temps qu’Einstein, les bases mathématiques de la relativité restreinte.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Science et l’Hypothèse&lt;/em&gt; (1902), il défend le &lt;a href="https://fr.wikipedia.org/wiki/Conventionnalisme" title=" Wikipedia"&gt;conventionnalisme&lt;/a&gt; : certains principes de la science ne sont ni des vérités a priori ni des faits d’expérience, mais des conventions. Ainsi, aucune expérience ne peut dire si l’espace est euclidien ou non : nous choisissons la géométrie d’Euclide parce qu’elle est la plus commode. Ces conventions ne sont pas arbitraires, car l’expérience nous guide, mais elles ne peuvent être ni vraies ni fausses. La science ne connaît pas les choses elles-mêmes, mais les rapports entre les choses.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;La Valeur de la science&lt;/em&gt; (1905) et &lt;em&gt;Science et méthode&lt;/em&gt; (1908), il s’oppose aussi aux logiciens, comme Russell, qui veulent réduire les mathématiques à la logique : pour lui, le raisonnement mathématique repose sur une intuition. Il décrit le rôle de l’inconscient dans la découverte, à partir de ses propres illuminations soudaines, comme celle qui lui vint en montant dans un omnibus. Élu à l’Académie française en 1908, il meurt à Paris en 1912.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H148" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/leonrobin-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/poincare-mini.webp</t>
         </is>
       </c>
       <c r="J148" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">metaphysique ; epistemologie</t>
+          <t xml:space="preserve">epistemologie ; logique</t>
         </is>
       </c>
       <c r="K148" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Platonisme</t>
+          <t xml:space="preserve">Conventionnalisme</t>
         </is>
       </c>
       <c r="L148" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">historien français de la philosophie grecque, grand interprète et traducteur de Platon.</t>
+          <t xml:space="preserve">mathématicien et physicien français, philosophe des sciences et fondateur du conventionnalisme.</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
@@ -9773,50 +9778,52 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
-      <c r="O148"/>
+      <c r="O148">
+        <v>2</v>
+      </c>
     </row>
     <row r="149" ht="176.25" customHeight="1" s="49">
       <c r="A149" s="47">
-        <v>1898</v>
+        <v>1866</v>
       </c>
       <c r="B149" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1994</t>
+          <t xml:space="preserve">1947</t>
         </is>
       </c>
       <c r="C149" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1898 – 1994</t>
+          <t xml:space="preserve">1866 – 1947</t>
         </is>
       </c>
       <c r="D149" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Henri GOUHIER</t>
+          <t xml:space="preserve">Léon ROBIN</t>
         </is>
       </c>
       <c r="E149" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Henri_Gouhier" title=" Wikipedia"&gt;Henri GOUHIER&lt;/a&gt; est un philosophe, historien de la philosophie et critique de théâtre français. Né à Auxerre en 1898, fils d’un clerc de notaire et d’une modiste, il entre à l’École normale supérieure en 1919 et est reçu premier à l’agrégation de philosophie en 1921. Élève d’&lt;a href="https://fr.wikipedia.org/wiki/%C3%89tienne_Gilson" title=" Wikipedia"&gt;Étienne Gilson&lt;/a&gt;, qui lui demande de faire pour la pensée française moderne ce qu’il fait lui-même pour le Moyen Âge, il enseigne à Lille, à Bordeaux, puis à la Sorbonne de 1941 à 1968, dans la chaire d’histoire de la pensée religieuse en France.&lt;/p&gt; &lt;p&gt;Il consacre sa vie à la philosophie française de Descartes à Bergson, qu’il lit en historien attentif aux convictions religieuses des auteurs. Il étudie la pensée religieuse de Descartes, Malebranche, Pascal, et surtout, dans trois volumes, la jeunesse d’Auguste Comte et la naissance du positivisme. Il montre comment le fondateur de la religion de l’Humanité a remplacé Dieu par l’humanité. Ces travaux inspirent le théologien Henri de Lubac pour &lt;em&gt;Le Drame de l’humanisme athée&lt;/em&gt; (1944). Il écrit aussi sur les conversions de Maine de Biran, sur Rousseau et sur Bergson, et défend l’idée d’une philosophie chrétienne.&lt;/p&gt; &lt;p&gt;Passionné de théâtre, il est pendant des décennies critique dramatique et publie &lt;em&gt;L’Essence du théâtre&lt;/em&gt; (1943), où il voit dans la représentation une présence réelle, une action vivante et non un simple texte. Membre de l’Académie des sciences morales et politiques, il est élu en 1979 à l’Académie française, au fauteuil de son maître Gilson. Il meurt à Paris en 1994.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/L%C3%A9on_Robin" title=" Wikipedia"&gt;Léon ROBIN&lt;/a&gt; est un philosophe et historien français de la philosophie, l’un des grands spécialistes de la pensée grecque. Né à Nantes en 1866, fils de marchand, il est reçu à l’agrégation de philosophie en 1891 et enseigne longtemps dans les lycées, à Compiègne, Vendôme et Angers. Élève et disciple d’Octave Hamelin, il publie après la mort de celui-ci son cours sur &lt;em&gt;Le Système d’Aristote&lt;/em&gt;. Il enseigne ensuite à Caen, puis à la Sorbonne de 1913 à 1937, où il occupe à partir de 1924 la chaire d’histoire de la philosophie antique.&lt;/p&gt; &lt;p&gt;Sa thèse, &lt;em&gt;La Théorie platonicienne des Idées et des nombres d’après Aristote&lt;/em&gt; (1908), s’appuie sur les témoignages d’Aristote pour reconstituer l’enseignement oral de &lt;a href="https://fr.wikipedia.org/wiki/Platon" title=" Wikipedia"&gt;Platon&lt;/a&gt; à l’Académie, où les Idées sont rattachées à des principes mathématiques, l’Un et la Dyade. Dans &lt;em&gt;La Pensée grecque et les origines de l’esprit scientifique&lt;/em&gt; (1923), il retrace la naissance de la raison grecque, des premiers physiciens d’Ionie jusqu’aux écoles hellénistiques. Il consacre aussi des livres à la morale antique, à Platon et au scepticisme de Pyrrhon, toujours appuyés sur une lecture rigoureuse des textes grecs.&lt;/p&gt; &lt;p&gt;Son œuvre la plus durable est la traduction des œuvres complètes de Platon pour la Bibliothèque de la Pléiade, qu’il dirige et dont il traduit lui-même la plus grande partie : précise et élégante, elle a fait lire Platon à des générations de lecteurs français. Il dirige aussi l’Institut international de philosophie. Il meurt à Paris en 1947. Pierre-Maxime Schuhl lui a succédé à la Sorbonne.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H149" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/gouhier-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/leonrobin-mini.webp</t>
         </is>
       </c>
       <c r="J149" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">metaphysique ; spiritualite ; esthetique</t>
+          <t xml:space="preserve">metaphysique ; epistemologie</t>
         </is>
       </c>
       <c r="K149" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spiritualisme ; Cartésianisme</t>
+          <t xml:space="preserve">Platonisme</t>
         </is>
       </c>
       <c r="L149" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">historien français de la philosophie, de Descartes à Bergson, et critique dramatique.</t>
+          <t xml:space="preserve">historien français de la philosophie grecque, grand interprète et traducteur de Platon.</t>
         </is>
       </c>
       <c r="N149" t="inlineStr">
@@ -9828,46 +9835,46 @@
     </row>
     <row r="150" ht="176.25" customHeight="1" s="49">
       <c r="A150" s="47">
-        <v>1918</v>
+        <v>1898</v>
       </c>
       <c r="B150" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1990</t>
+          <t xml:space="preserve">1994</t>
         </is>
       </c>
       <c r="C150" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1918 – 1990</t>
+          <t xml:space="preserve">1898 – 1994</t>
         </is>
       </c>
       <c r="D150" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Henri BIRAULT</t>
+          <t xml:space="preserve">Henri GOUHIER</t>
         </is>
       </c>
       <c r="E150" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Henri_Birault" title=" Wikipedia"&gt;Henri BIRAULT&lt;/a&gt; est un philosophe français. Né à Paris en 1918, il entre à l’École normale supérieure en 1939, dans la même promotion que Louis Althusser et Jules Vuillemin, et est reçu deuxième à l’agrégation de philosophie en 1945. Élève de Louis Lavelle et de Jean Nabert, il découvre ensuite l’œuvre de &lt;a href="https://fr.wikipedia.org/wiki/Martin_Heidegger" title=" Wikipedia"&gt;Martin Heidegger&lt;/a&gt;, dont il devient, avec Jean Beaufret, l’un des grands commentateurs français. Il enseigne en khâgne au lycée Henri-IV, puis à la Sorbonne.&lt;/p&gt; &lt;p&gt;Professeur admiré, il marque plusieurs générations d’étudiants par ses lectures lentes et minutieuses des textes, qu’il lit dans leur langue d’origine, en grec, en latin, en allemand. Sa réflexion, nourrie de Pascal, de Kant, de Nietzsche et de Heidegger, porte sur la question de l’être et sur la finitude humaine. Avec Heidegger, il cherche à comprendre ce que veut dire penser, au-delà de la métaphysique qui a réduit l’être à un objet disponible pour la science et la technique. Il en tire &lt;em&gt;Heidegger et l’expérience de la pensée&lt;/em&gt; (1978), qui reste l’une des grandes introductions françaises à cette œuvre difficile.&lt;/p&gt; &lt;p&gt;Sa contribution la plus célèbre, « De la béatitude chez Nietzsche », présentée en 1964 au colloque de Royaumont, montre que Nietzsche n’est pas seulement le penseur de la volonté de puissance et de la mort de Dieu, mais aussi celui d’une joie, d’une approbation sans réserve de la vie, de l’« amour du destin ». Respecté par Deleuze et ses contemporains, il publie peu et réécrit sans cesse. Il meurt en 1990. &lt;em&gt;De l’Être, du divin et des dieux&lt;/em&gt; paraît en 2005.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Henri_Gouhier" title=" Wikipedia"&gt;Henri GOUHIER&lt;/a&gt; est un philosophe, historien de la philosophie et critique de théâtre français. Né à Auxerre en 1898, fils d’un clerc de notaire et d’une modiste, il entre à l’École normale supérieure en 1919 et est reçu premier à l’agrégation de philosophie en 1921. Élève d’&lt;a href="https://fr.wikipedia.org/wiki/%C3%89tienne_Gilson" title=" Wikipedia"&gt;Étienne Gilson&lt;/a&gt;, qui lui demande de faire pour la pensée française moderne ce qu’il fait lui-même pour le Moyen Âge, il enseigne à Lille, à Bordeaux, puis à la Sorbonne de 1941 à 1968, dans la chaire d’histoire de la pensée religieuse en France.&lt;/p&gt; &lt;p&gt;Il consacre sa vie à la philosophie française de Descartes à Bergson, qu’il lit en historien attentif aux convictions religieuses des auteurs. Il étudie la pensée religieuse de Descartes, Malebranche, Pascal, et surtout, dans trois volumes, la jeunesse d’Auguste Comte et la naissance du positivisme. Il montre comment le fondateur de la religion de l’Humanité a remplacé Dieu par l’humanité. Ces travaux inspirent le théologien Henri de Lubac pour &lt;em&gt;Le Drame de l’humanisme athée&lt;/em&gt; (1944). Il écrit aussi sur les conversions de Maine de Biran, sur Rousseau et sur Bergson, et défend l’idée d’une philosophie chrétienne.&lt;/p&gt; &lt;p&gt;Passionné de théâtre, il est pendant des décennies critique dramatique et publie &lt;em&gt;L’Essence du théâtre&lt;/em&gt; (1943), où il voit dans la représentation une présence réelle, une action vivante et non un simple texte. Membre de l’Académie des sciences morales et politiques, il est élu en 1979 à l’Académie française, au fauteuil de son maître Gilson. Il meurt à Paris en 1994.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H150" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/birault-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/gouhier-mini.webp</t>
         </is>
       </c>
       <c r="J150" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">metaphysique ; spiritualite</t>
+          <t xml:space="preserve">metaphysique ; spiritualite ; esthetique</t>
         </is>
       </c>
       <c r="K150" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phénoménologie</t>
+          <t xml:space="preserve">Spiritualisme ; Cartésianisme</t>
         </is>
       </c>
       <c r="L150" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe français, grand lecteur de Heidegger, de Nietzsche et de Pascal.</t>
+          <t xml:space="preserve">historien français de la philosophie, de Descartes à Bergson, et critique dramatique.</t>
         </is>
       </c>
       <c r="N150" t="inlineStr">
@@ -9879,51 +9886,46 @@
     </row>
     <row r="151" ht="176.25" customHeight="1" s="49">
       <c r="A151" s="47">
-        <v>1923</v>
+        <v>1918</v>
       </c>
       <c r="B151" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">2007</t>
+          <t xml:space="preserve">1990</t>
         </is>
       </c>
       <c r="C151" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1923 – 2007</t>
+          <t xml:space="preserve">1918 – 1990</t>
         </is>
       </c>
       <c r="D151" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">André GORZ</t>
+          <t xml:space="preserve">Henri BIRAULT</t>
         </is>
       </c>
       <c r="E151" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Andr%C3%A9_Gorz" title=" Wikipedia"&gt;André GORZ&lt;/a&gt; est un philosophe et journaliste français d’origine autrichienne, l’un des fondateurs de l’écologie politique. Né Gerhart Hirsch à Vienne en 1923, d’un père juif et d’une mère catholique, il est envoyé en Suisse en 1939 pour échapper à la guerre et y devient ingénieur chimiste. En 1946, il rencontre &lt;a href="https://fr.wikipedia.org/wiki/Jean-Paul_Sartre" title=" Wikipedia"&gt;Jean-Paul Sartre&lt;/a&gt;, qui le marque profondément. Installé à Paris en 1949, il écrit sous le nom de Michel Bosquet pour &lt;em&gt;L’Express&lt;/em&gt;, puis participe en 1964 à la fondation du &lt;em&gt;Nouvel Observateur&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Traître&lt;/em&gt; (1958), préfacé par Sartre, il analyse sa propre vie en existentialiste. Penseur du marxisme critique, il s’intéresse ensuite au travail : dans &lt;em&gt;Adieux au prolétariat&lt;/em&gt; (1980), il affirme que la classe ouvrière n’est plus le sujet de l’émancipation, et que la libération passe par la réduction du temps de travail. L’automatisation permettrait de travailler beaucoup moins, et de développer les activités libres, choisies pour elles-mêmes, plutôt que de produire et consommer toujours plus.&lt;/p&gt; &lt;p&gt;Dès &lt;em&gt;Écologie et politique&lt;/em&gt; (1975), il relie la crise écologique au capitalisme : la croissance infinie détruit la nature et les liens humains. L’écologie doit être une politique de l’autonomie, qui permette de « produire moins, vivre mieux ». Il défendra plus tard un revenu d’existence versé à tous, indépendamment de l’emploi. Dans &lt;em&gt;Lettre à D.&lt;/em&gt; (2006), il écrit un émouvant livre d’amour à sa femme Dorine, gravement malade. Ils se donnent la mort ensemble en 2007, dans leur maison de Vosnon, dans l’Aube.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Henri_Birault" title=" Wikipedia"&gt;Henri BIRAULT&lt;/a&gt; est un philosophe français. Né à Paris en 1918, il entre à l’École normale supérieure en 1939, dans la même promotion que Louis Althusser et Jules Vuillemin, et est reçu deuxième à l’agrégation de philosophie en 1945. Élève de Louis Lavelle et de Jean Nabert, il découvre ensuite l’œuvre de &lt;a href="https://fr.wikipedia.org/wiki/Martin_Heidegger" title=" Wikipedia"&gt;Martin Heidegger&lt;/a&gt;, dont il devient, avec Jean Beaufret, l’un des grands commentateurs français. Il enseigne en khâgne au lycée Henri-IV, puis à la Sorbonne.&lt;/p&gt; &lt;p&gt;Professeur admiré, il marque plusieurs générations d’étudiants par ses lectures lentes et minutieuses des textes, qu’il lit dans leur langue d’origine, en grec, en latin, en allemand. Sa réflexion, nourrie de Pascal, de Kant, de Nietzsche et de Heidegger, porte sur la question de l’être et sur la finitude humaine. Avec Heidegger, il cherche à comprendre ce que veut dire penser, au-delà de la métaphysique qui a réduit l’être à un objet disponible pour la science et la technique. Il en tire &lt;em&gt;Heidegger et l’expérience de la pensée&lt;/em&gt; (1978), qui reste l’une des grandes introductions françaises à cette œuvre difficile.&lt;/p&gt; &lt;p&gt;Sa contribution la plus célèbre, « De la béatitude chez Nietzsche », présentée en 1964 au colloque de Royaumont, montre que Nietzsche n’est pas seulement le penseur de la volonté de puissance et de la mort de Dieu, mais aussi celui d’une joie, d’une approbation sans réserve de la vie, de l’« amour du destin ». Respecté par Deleuze et ses contemporains, il publie peu et réécrit sans cesse. Il meurt en 1990. &lt;em&gt;De l’Être, du divin et des dieux&lt;/em&gt; paraît en 2005.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H151" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/gorz-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/birault-mini.webp</t>
         </is>
       </c>
       <c r="J151" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">politique ; ethique</t>
+          <t xml:space="preserve">metaphysique ; spiritualite</t>
         </is>
       </c>
       <c r="K151" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ecologisme ; Marxisme</t>
+          <t xml:space="preserve">Phénoménologie</t>
         </is>
       </c>
       <c r="L151" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe et journaliste français, l’un des fondateurs de l’écologie politique.</t>
-        </is>
-      </c>
-      <c r="M151" t="inlineStr">
-        <is>
-          <t xml:space="preserve">juive</t>
+          <t xml:space="preserve">philosophe français, grand lecteur de Heidegger, de Nietzsche et de Pascal.</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
@@ -9931,52 +9933,55 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
-      <c r="O151">
-        <v>2</v>
-      </c>
+      <c r="O151"/>
     </row>
     <row r="152" ht="176.25" customHeight="1" s="49">
       <c r="A152" s="47">
-        <v>1936</v>
+        <v>1923</v>
       </c>
       <c r="B152" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025</t>
+          <t xml:space="preserve">2007</t>
         </is>
       </c>
       <c r="C152" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1936 – 2025</t>
+          <t xml:space="preserve">1923 – 2007</t>
         </is>
       </c>
       <c r="D152" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alain ROGER</t>
+          <t xml:space="preserve">André GORZ</t>
         </is>
       </c>
       <c r="E152" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Alain_Roger" title=" Wikipedia"&gt;Alain ROGER&lt;/a&gt; est un philosophe et écrivain français. Né à Mirecourt, dans les Vosges, en 1936, ancien élève de l’École normale supérieure, agrégé de philosophie et élève de &lt;a href="https://fr.wikipedia.org/wiki/Gilles_Deleuze" title=" Wikipedia"&gt;Gilles Deleuze&lt;/a&gt;, il enseigne l’esthétique à l’université de Clermont-Ferrand. Romancier, il publie notamment &lt;em&gt;La Travestie&lt;/em&gt; (1987), adaptée au cinéma par Yves Boisset. Mais il est surtout connu comme le grand théoricien français du &lt;a href="https://fr.wikipedia.org/wiki/Paysage" title=" Wikipedia"&gt;paysage&lt;/a&gt;, auquel il consacre l’essentiel de son œuvre de philosophe.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Nus et paysages&lt;/em&gt; (1978) puis dans le &lt;em&gt;Court traité du paysage&lt;/em&gt; (1997), il soutient que la beauté de la nature n’est pas naturelle : nous voyons le monde à travers les œuvres d’art. Il reprend à Montaigne le mot « artialisation » pour désigner cette transformation de la nature par l’art. Elle peut être directe, « in situ », quand on façonne un jardin ou un corps, ou indirecte, « in visu », quand la peinture, la poésie ou la photographie éduquent notre regard. Le paysage naît ainsi au XVe siècle dans la peinture flamande, par la « fenêtre » ouverte au fond des tableaux.&lt;/p&gt; &lt;p&gt;Il montre que des lieux longtemps jugés affreux, comme la montagne ou le bord de mer, ne sont devenus beaux qu’au XVIIIe siècle, grâce aux écrivains et aux peintres. Ses travaux inspirent paysagistes et aménageurs, et il enseigne à l’école d’architecture de Paris-La Villette. Il est aussi l’auteur d’un &lt;em&gt;Bréviaire de la bêtise&lt;/em&gt; (2008), recueil d’aphorismes sur la sottise et ses formes les plus savantes. Il meurt à Belley, dans l’Ain, le 7 octobre 2025.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Andr%C3%A9_Gorz" title=" Wikipedia"&gt;André GORZ&lt;/a&gt; est un philosophe et journaliste français d’origine autrichienne, l’un des fondateurs de l’écologie politique. Né Gerhart Hirsch à Vienne en 1923, d’un père juif et d’une mère catholique, il est envoyé en Suisse en 1939 pour échapper à la guerre et y devient ingénieur chimiste. En 1946, il rencontre &lt;a href="https://fr.wikipedia.org/wiki/Jean-Paul_Sartre" title=" Wikipedia"&gt;Jean-Paul Sartre&lt;/a&gt;, qui le marque profondément. Installé à Paris en 1949, il écrit sous le nom de Michel Bosquet pour &lt;em&gt;L’Express&lt;/em&gt;, puis participe en 1964 à la fondation du &lt;em&gt;Nouvel Observateur&lt;/em&gt;.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Le Traître&lt;/em&gt; (1958), préfacé par Sartre, il analyse sa propre vie en existentialiste. Penseur du marxisme critique, il s’intéresse ensuite au travail : dans &lt;em&gt;Adieux au prolétariat&lt;/em&gt; (1980), il affirme que la classe ouvrière n’est plus le sujet de l’émancipation, et que la libération passe par la réduction du temps de travail. L’automatisation permettrait de travailler beaucoup moins, et de développer les activités libres, choisies pour elles-mêmes, plutôt que de produire et consommer toujours plus.&lt;/p&gt; &lt;p&gt;Dès &lt;em&gt;Écologie et politique&lt;/em&gt; (1975), il relie la crise écologique au capitalisme : la croissance infinie détruit la nature et les liens humains. L’écologie doit être une politique de l’autonomie, qui permette de « produire moins, vivre mieux ». Il défendra plus tard un revenu d’existence versé à tous, indépendamment de l’emploi. Dans &lt;em&gt;Lettre à D.&lt;/em&gt; (2006), il écrit un émouvant livre d’amour à sa femme Dorine, gravement malade. Ils se donnent la mort ensemble en 2007, dans leur maison de Vosnon, dans l’Aube.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H152" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/alainroger-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/gorz-mini.webp</t>
         </is>
       </c>
       <c r="J152" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique</t>
+          <t xml:space="preserve">politique ; ethique</t>
         </is>
       </c>
       <c r="K152" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constructivisme</t>
+          <t xml:space="preserve">Ecologisme ; Marxisme</t>
         </is>
       </c>
       <c r="L152" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe et romancier français, théoricien de l’« artialisation » et de l’invention du paysage.</t>
+          <t xml:space="preserve">philosophe et journaliste français, l’un des fondateurs de l’écologie politique.</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">juive</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
@@ -9984,50 +9989,52 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
-      <c r="O152"/>
+      <c r="O152">
+        <v>2</v>
+      </c>
     </row>
     <row r="153" ht="176.25" customHeight="1" s="49">
       <c r="A153" s="47">
-        <v>1938</v>
+        <v>1936</v>
       </c>
       <c r="B153" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">2021</t>
+          <t xml:space="preserve">2025</t>
         </is>
       </c>
       <c r="C153" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1938 – 2021</t>
+          <t xml:space="preserve">1936 – 2025</t>
         </is>
       </c>
       <c r="D153" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pierre RABHI</t>
+          <t xml:space="preserve">Alain ROGER</t>
         </is>
       </c>
       <c r="E153" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pierre_Rabhi" title=" Wikipedia"&gt;Pierre RABHI&lt;/a&gt; est un agriculteur, essayiste et militant français, l’une des figures de l’&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cologisme" title=" Wikipedia"&gt;écologie&lt;/a&gt; en France. Né Rabah Rabhi en 1938 à Kenadsa, une oasis du sud de l’Algérie, il perd sa mère très jeune et est confié à un couple de Français d’Oran ; il se convertit au catholicisme et prend le prénom de Pierre. Venu à Paris, il travaille comme ouvrier, puis s’installe en 1961 avec sa femme Michèle dans les Cévennes ardéchoises, où il devient paysan et pratique une agriculture sans produits chimiques.&lt;/p&gt; &lt;p&gt;À partir de 1981, il forme des paysans au Burkina Faso, puis dans d’autres pays d’Afrique, à l’« agroécologie », une agriculture qui respecte les sols et rend les communautés autonomes. Dans ses livres, comme &lt;em&gt;Vers la sobriété heureuse&lt;/em&gt; (2010), il critique la société de consommation et l’idéologie de la croissance : il faut apprendre à vivre avec moins pour être plus heureux. En 2007, il fonde le mouvement Colibris, d’après une légende amérindienne : pendant un incendie de forêt, le colibri apporte des gouttes d’eau dans son bec, car il « fait sa part ».&lt;/p&gt; &lt;p&gt;Très populaire, il est candidat à l’élection présidentielle de 2002, sans réunir les signatures nécessaires. Son discours spirituel, sa proximité avec l’anthroposophie et son peu d’intérêt pour les combats politiques lui valent aussi des critiques, notamment de journalistes et de scientifiques qui contestent certaines de ses affirmations sur l’agriculture. Il meurt à Lyon en 2021. Son appel à une « insurrection des consciences » a inspiré de nombreuses initiatives locales d’écologie.&lt;/p&gt;</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Alain_Roger" title=" Wikipedia"&gt;Alain ROGER&lt;/a&gt; est un philosophe et écrivain français. Né à Mirecourt, dans les Vosges, en 1936, ancien élève de l’École normale supérieure, agrégé de philosophie et élève de &lt;a href="https://fr.wikipedia.org/wiki/Gilles_Deleuze" title=" Wikipedia"&gt;Gilles Deleuze&lt;/a&gt;, il enseigne l’esthétique à l’université de Clermont-Ferrand. Romancier, il publie notamment &lt;em&gt;La Travestie&lt;/em&gt; (1987), adaptée au cinéma par Yves Boisset. Mais il est surtout connu comme le grand théoricien français du &lt;a href="https://fr.wikipedia.org/wiki/Paysage" title=" Wikipedia"&gt;paysage&lt;/a&gt;, auquel il consacre l’essentiel de son œuvre de philosophe.&lt;/p&gt; &lt;p&gt;Dans &lt;em&gt;Nus et paysages&lt;/em&gt; (1978) puis dans le &lt;em&gt;Court traité du paysage&lt;/em&gt; (1997), il soutient que la beauté de la nature n’est pas naturelle : nous voyons le monde à travers les œuvres d’art. Il reprend à Montaigne le mot « artialisation » pour désigner cette transformation de la nature par l’art. Elle peut être directe, « in situ », quand on façonne un jardin ou un corps, ou indirecte, « in visu », quand la peinture, la poésie ou la photographie éduquent notre regard. Le paysage naît ainsi au XVe siècle dans la peinture flamande, par la « fenêtre » ouverte au fond des tableaux.&lt;/p&gt; &lt;p&gt;Il montre que des lieux longtemps jugés affreux, comme la montagne ou le bord de mer, ne sont devenus beaux qu’au XVIIIe siècle, grâce aux écrivains et aux peintres. Ses travaux inspirent paysagistes et aménageurs, et il enseigne à l’école d’architecture de Paris-La Villette. Il est aussi l’auteur d’un &lt;em&gt;Bréviaire de la bêtise&lt;/em&gt; (2008), recueil d’aphorismes sur la sottise et ses formes les plus savantes. Il meurt à Belley, dans l’Ain, le 7 octobre 2025.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H153" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/rabhi-mini.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/alainroger-mini.webp</t>
         </is>
       </c>
       <c r="J153" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">ethique ; politique ; spiritualite</t>
+          <t xml:space="preserve">esthetique</t>
         </is>
       </c>
       <c r="K153" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ecologisme</t>
+          <t xml:space="preserve">Constructivisme</t>
         </is>
       </c>
       <c r="L153" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">agriculteur et essayiste français, pionnier de l’agroécologie et chantre de la « sobriété heureuse ».</t>
+          <t xml:space="preserve">philosophe et romancier français, théoricien de l’« artialisation » et de l’invention du paysage.</t>
         </is>
       </c>
       <c r="N153" t="inlineStr">
@@ -10039,55 +10046,46 @@
     </row>
     <row r="154" ht="176.25" customHeight="1" s="49">
       <c r="A154" s="47">
-        <v>1937</v>
-      </c>
-      <c r="B154" s="47">
-        <v>2026</v>
+        <v>1938</v>
+      </c>
+      <c r="B154" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2021</t>
+        </is>
       </c>
       <c r="C154" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">1937 – 2026</t>
+          <t xml:space="preserve">1938 – 2021</t>
         </is>
       </c>
       <c r="D154" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Éliane ESCOUBAS</t>
+          <t xml:space="preserve">Pierre RABHI</t>
         </is>
       </c>
       <c r="E154" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/%C3%89liane_Escoubas"  style="color:#6A142A"  title=" Wikipedia"&gt;Éliane ESCOUBAS&lt;/a&gt;  est une philosophe française, historienne de la philosophie et traductrice. Elle se rattache à l’école phénoménologique et travaille principalement sur la philosophie allemande, la phénoménologie de l’art et la psychiatrie phénoménologique, dite Daseinsanalyse. Après une formation marquée par les cours de Gérard Granel sur Husserl, Kant et Hegel à Toulouse, elle enseigne dans le secondaire puis devient maître de conférences, puis professeur de philosophie, tout en menant des recherches au CNRS et en participant à la création du Collège international de Philosophie. &lt;/p&gt; &lt;p&gt; Elle met au centre la phénoménologie de l’expérience sensible, en particulier la manière dont le monde et le sujet adviennent à travers le sentir, l’affect et la perception. Elle montre que la phénoménologie fournit un prisme particulièrement adapté pour penser l’esthétique, car l’œuvre d’art apparaît comme un mode privilégié pour saisir comment le sujet et le monde se co‑constituent dans une expérience sensible et existentielle. &lt;/p&gt; &lt;p&gt; Une grande partie de son œuvre est consacrée à une « esthétique du sentir » où l’art n’est pas seulement une illustration de la philosophie, mais un mode de connaissance autonome. Dans ses travaux comme Imago mundi. Topologie de l’art ou L’invention de l’art, elle montre que l’image et l’œuvre picturale ne se réduisent pas à « représentation » ou « signe », mais relèvent d’une apparition du monde lui‑même, d’une spatialité et d’une temporalité qui précèdent les catégories classiques de l’objet. &lt;/p&gt; &lt;p&gt; Sa philosophie s’ouvre aussi à la phénoménologie clinique et à la psychiatrie, notamment à travers la Daseinsanalyse et la place de l’affect et de l’affectivité dans la constitution du sujet. En explorant les affectivités dans la modernité et la phénoménologie, Escoubas prolonge ainsi une réflexion sur la manière dont le vécu, le corps et la subjectivité forment un champ de savoir propre, à la fois esthétique, analytique et existentiel. Elle meurt à Paris le 18 juillet 2026. &lt;/p&gt;  &lt;audio controls title="Alain BADIOU par France Culture"&gt; &lt;source src="https://media.radiofrance-podcast.net/podcast09/10080-25.11.2011-ITEMA_20320112-2011C3403E0190-ITE_00047070_RSCE-21.mp3" type="audio/mpeg" align="center"&gt; &lt;/audio&gt; 
-</t>
+          <t xml:space="preserve">&lt;p&gt;&lt;a href="https://fr.wikipedia.org/wiki/Pierre_Rabhi" title=" Wikipedia"&gt;Pierre RABHI&lt;/a&gt; est un agriculteur, essayiste et militant français, l’une des figures de l’&lt;a href="https://fr.wikipedia.org/wiki/%C3%89cologisme" title=" Wikipedia"&gt;écologie&lt;/a&gt; en France. Né Rabah Rabhi en 1938 à Kenadsa, une oasis du sud de l’Algérie, il perd sa mère très jeune et est confié à un couple de Français d’Oran ; il se convertit au catholicisme et prend le prénom de Pierre. Venu à Paris, il travaille comme ouvrier, puis s’installe en 1961 avec sa femme Michèle dans les Cévennes ardéchoises, où il devient paysan et pratique une agriculture sans produits chimiques.&lt;/p&gt; &lt;p&gt;À partir de 1981, il forme des paysans au Burkina Faso, puis dans d’autres pays d’Afrique, à l’« agroécologie », une agriculture qui respecte les sols et rend les communautés autonomes. Dans ses livres, comme &lt;em&gt;Vers la sobriété heureuse&lt;/em&gt; (2010), il critique la société de consommation et l’idéologie de la croissance : il faut apprendre à vivre avec moins pour être plus heureux. En 2007, il fonde le mouvement Colibris, d’après une légende amérindienne : pendant un incendie de forêt, le colibri apporte des gouttes d’eau dans son bec, car il « fait sa part ».&lt;/p&gt; &lt;p&gt;Très populaire, il est candidat à l’élection présidentielle de 2002, sans réunir les signatures nécessaires. Son discours spirituel, sa proximité avec l’anthroposophie et son peu d’intérêt pour les combats politiques lui valent aussi des critiques, notamment de journalistes et de scientifiques qui contestent certaines de ses affirmations sur l’agriculture. Il meurt à Lyon en 2021. Son appel à une « insurrection des consciences » a inspiré de nombreuses initiatives locales d’écologie.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="H154" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">https://www.laphilo.fr/pho/eescoubas-mini.webp</t>
-        </is>
-      </c>
-      <c r="I154" t="inlineStr">
-        <is>
-          <t xml:space="preserve">https://laphilo.fr/photo/escoubas.webp</t>
+          <t xml:space="preserve">https://www.laphilo.fr/pho/rabhi-mini.webp</t>
         </is>
       </c>
       <c r="J154" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">esthetique ; epistemologie</t>
+          <t xml:space="preserve">ethique ; politique ; spiritualite</t>
         </is>
       </c>
       <c r="K154" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phénoménologie</t>
+          <t xml:space="preserve">Ecologisme</t>
         </is>
       </c>
       <c r="L154" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">philosophe française, historienne de la philosophie et traductrice.</t>
-        </is>
-      </c>
-      <c r="M154" t="inlineStr">
-        <is>
-          <t xml:space="preserve">femme</t>
+          <t xml:space="preserve">agriculteur et essayiste français, pionnier de l’agroécologie et chantre de la « sobriété heureuse ».</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
@@ -10095,6 +10093,7 @@
           <t xml:space="preserve">occident</t>
         </is>
       </c>
+      <c r="O154"/>
     </row>
     <row r="1048566" ht="12.75" customHeight="1" s="49"/>
     <row r="1048567" ht="12.75" customHeight="1" s="49"/>
@@ -10195,30 +10194,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H126" display="https://www.laphilo.fr/pho/mwittig-mini.webp" r:id="rId79"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E127" display=" &lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Michel_Hulin&quot;  title=&quot; Wikipedia&quot;&gt;Michel HULIN&lt;/a&gt; était un philosophe français récemment décédé, grand spécialiste de la &lt;a href=&quot;https://www.youtube.com/watch?v=tJFic9y58Sc&quot; title=&quot; Aperçu de l’hindouisme avec Michel Hulin par Resonances &quot;&gt;philosophie indienne &lt;/a&gt; et de la comparaison entre pensée européenne et pensée asiatique, notamment de l’Advaïta Vedānta, le courant « non‑dualiste » du vedānta. Longtemps professeur de philosophie indienne et comparée à l’université Paris‑Sorbonne, il a joué un rôle central dans la diffusion en France des grandes écoles de pensée de l’Inde. Sa carrière s’est accompagnée d’un important travail de traduction du sanskrit et de vulgarisation, accessible à un public non spécialiste. &lt;/p&gt; &lt;p&gt; Ses recherches portent d’une part sur  &lt;a href=&quot;https://www.youtube.com/watch?v=kaJP8yDwHeY&quot; title=&quot; For intérieur par Resonnances &quot;&gt;la pensée indienne classique &lt;/a&gt;  (notion d’ahamkāra, textes vedāntins et shivaïtes d’inspiration tantrique), d’autre part sur les questions épistémologiques et métaphysiques que soulève la rencontre entre les traditions européennes et asiatiques. Dans sa thèse, Le Principe de l’ego dans la pensée indienne classique, il analyse la notion de « faux moi » et montre comment elle éclaire notre expérience ordinaire de la conscience. Il s’intéresse également à la question du temps, de l’éternité et des expériences dites mystiques, qu’il relie à des vécus très concrets. &lt;/p&gt; &lt;p&gt; Dans des ouvrages comme La Face cachée du temps, La Mystique sauvage, Hegel et l’Orient, Shankara et la non‑dualité ou encore l’anthologie L’Inde des sages, il  conjugue une érudition très précise et un style volontairement clair. Il montre comment des interrogations métaphysiques complexes – sur le moi, le temps, l’au‑delà ou l’expérience spirituelle – touchent directement la vie intérieure de chacun. Par son enseignement et ses livres, il a contribué à installer durablement en France une philosophie comparée attentive au dialogue entre Europe et Inde. &lt;p&gt; &lt;/p&gt;&lt;audio controls title=&quot;  Philosophies indiennes (1/4) : Upanishads, les textes fondateurs ?  par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10467-16.12.2013-ITEMA_20562153-2013C12410S0350-NET_FC_A092AF0E-5BC1-49EE-A72F-E62BB6A2A8B1-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  &lt;p&gt;  &lt;/p&gt;&#10;" r:id="rId80"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H127" display="https://www.laphilo.fr/pho/mhulin-mini.webp" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H128" display="https://www.laphilo.fr/pho/jfmarquet-mini.webp" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E129" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Cl%C3%A9ment_Rosset&quot; title=&quot; Wikipedia&quot;&gt;Clément ROSSET&lt;/a&gt; était un philosophe français connu pour sa pensée radicale et son style d'écriture d'une grande clarté. Son œuvre est principalement centrée sur le concept du  &lt;a href=&quot;https://www.youtube.com/watch?v=I50Jbj6uQEU&quot; title=&quot;Clément Rosset : la réalité ne convient pas ! par Kosmos&quot;&gt;&quot;réel&quot;&lt;/a&gt;  et l'incapacité ou la difficulté de l'homme à l'accepter dans sa singularité et souvent sa cruauté. Voici les points essentiels concernant sa philosophie : &lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.youtube.com/watch?v=8m_kXVBdtwg&quot;  title=&quot; Le réel et son double, Clément Rosset, 2.2 avant-propos par Thibault BELZACQ&quot;&gt;Le Réel sans double&lt;/a&gt; : Son idée maîtresse est que le réel est unique, singulier et dépourvu de tout &quot;double&quot;. Il n'y a pas d'arrière-monde, pas de sens caché, pas de consolation ou d'illusion qui puisse atténuer sa nature brute. Le réel est simplement ce qui est, dans son évidence la plus nue. &lt;/p&gt; &lt;p&gt; - Le Refus du double et de l'illusion : Une grande partie de son travail consiste à traquer les différentes formes d'illusions et de doubles que l'humanité crée pour  &lt;a href=&quot;https://philitt.fr/2023/09/12/clement-rosset-tout-est-sans-raison/&quot;  title=&quot;Clément Rosset : tout est sans raison par Phillitt&quot;&gt;échapper à la confrontation&lt;/a&gt; directe avec le réel. Ces doubles peuvent être d'ordre métaphysique, moral, psychologique, ou même esthétique.&lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.youtube.com/watch?v=JDcudFE_uBQ&quot;  title=&quot;Entretien avec Pierre Dumayet (1961) par Archives&quot;&gt;Philosophie tragique&lt;/a&gt; et Joie : Bien que sa pensée puisse sembler sombre en insistant sur la cruauté et l'absurdité du réel, il développe une philosophie que l'on qualifie souvent de &quot;tragique&quot; au sens nietzschéen du terme. Il ne s'agit pas de désespoir, mais plutôt de l'affirmation de la vie et du réel tels qu'ils sont, y compris dans leurs aspects les plus difficiles. &lt;/p&gt; &lt;p&gt; Il est également remarquable par son style d'écriture. Loin du jargon philosophique abscons, il privilégie une langue simple, directe et percutante. Cette clarté formelle est au service de la clarté de sa pensée, cherchant à énoncer le réel avec le moins d'interférences possible. Son œuvre, bien que parfois restée en marge des courants universitaires dominants, a marqué par sa radicalité, sa lucidité et sa défense d'une confrontation sans fard avec le réel.  &lt;/p&gt; &lt;audio controls title=&quot;Clément Rosset par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10080-20.12.2013-ITEMA_20564152-2013C3403E0215-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  " r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" display="https://www.laphilo.fr/pho/rosset-mini.webp" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Jacques_Bouveresse&quot;  title=&quot; Wikipedia&quot;&gt;Jacques BOUVERESSE&lt;/a&gt; était un philosophe français du courant analytique, connu pour son rationalisme exigeant, son &lt;a href=&quot;https://www.youtube.com/watch?v=mfGM00nmj20&quot;  title=&quot; Wittgenstein et l'intériorité 一 Jacques Bouveresse par Andrea Cirla &quot;&gt;travail sur Wittgenstein &lt;/a&gt; et sa critique des dérives du milieu intellectuel français. Il a largement contribué à introduire et stabiliser en France une philosophie soucieuse de vérité, de clarté et d’argumentation rigoureuse. &lt;/p&gt; &lt;p&gt; Ses domaines privilégiés sont la philosophie de la connaissance, des sciences, des mathématiques, de la logique, du langage, ainsi qu’une philosophie de la culture attentive à la littérature et à la critique sociale.  Il se réclame du rationalisme des Lumières et s’inspire fortement de la philosophie analytique, du Cercle de Vienne, de Frege, de Gödel et de la tradition d’Europe centrale. Wittgenstein, qu’il contribue à faire connaître en France, est l’une de ses références centrales. &lt;/p&gt; &lt;p&gt; Il défend une position rationaliste dont le prolongement éthique est ce qu’il appelle la  &lt;a href=&quot;https://www.persee.fr/doc/lgge_0458-726x_1971_num_6_21_2079&quot; title=&quot;Langage ordinaire et philosophie par Persée &quot;&gt;&quot;modestie intellectuelle&quot; &lt;/a&gt; : ne pas exagérer ce que la philosophie peut faire, refuser le pathos et le prestige facile. Il combat le relativisme, l’historicisme radical et les remises en cause globales de la notion de vérité, notamment chez certains auteurs français, tout en reconnaissant par ailleurs leur importance. &lt;/p&gt; &lt;p&gt; Sa grande thèse, &quot;Le Mythe de l’intériorité&quot;, porte sur Wittgenstein, le langage privé, l’expérience et la signification, et a joué un rôle clé dans la réception française de Wittgenstein. Il consacre de nombreux travaux à Robert Musil et Karl Kraus, qu’il lit comme des alliés dans un combat pour l’exactitude, la critique de la bêtise et des illusions de la culture moderne. &lt;/p&gt;  &lt;audio controls title=&quot;Jacques Bouveresse, à la recherche de la clarté par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10351-11.05.2021-ITEMA_23961779-2000C3500E0287-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" display="https://www.laphilo.fr/pho/bouveresse-mini.webp" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Jean-Luc_Nancy&quot;  title=&quot; Wikipedia&quot;&gt;Jean-Luc NANCY&lt;/a&gt; était un philosophe français, agrégé de philosophie, il fut professeur à l'Université de Strasbourg jusqu'à sa retraite. Sa pensée, en dialogue constant avec Heidegger, Derrida et Lacoue-Labarthe — avec lequel il collabora étroitement — porte sur le « sens du monde », la communauté, le corps et le toucher. &lt;/p&gt; &lt;p&gt; Son œuvre est marquée par le questionnement du « with » (avec), du « being-with » heideggerien. Dans &lt;em&gt;La Communauté désoeuvrée&lt;/em&gt; (1986), il développe une pensée de la communauté qui refuse toute forme d'immanentisme ou de fusion : la communauté véritable n'est pas une substance commune, mais  &lt;a href=&quot;https://www.youtube.com/watch?v=fZK6pEAPxEw&quot;  title=&quot;jean luc Nancy par Institut Humanités &quot;&gt;l'exposition partagée &lt;/a&gt; de la singularité de chacun. Cette réflexion, en dialogue critique avec Blanchot et Bataille, a eu un retentissement considérable dans les débats contemporains sur la politique, la communauté et l'identité. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Corpus&lt;/em&gt; (1992) et &lt;em&gt;Noli me tangere&lt;/em&gt; (2003), il explore  &lt;a href=&quot;https://www.youtube.com/watch?v=1kCExw6Wp9k&quot;  title=&quot;jean luc Nancy par Lacan TV &quot;&gt;la philosophie du corps &lt;/a&gt; et du toucher comme modes fondamentaux de l'être-au-monde. Son essai sur le sens — &lt;em&gt;Le Sens du monde&lt;/em&gt; (1993) — aborde la question de la possibilité du sens dans un monde déserté par les transcendances. &lt;em&gt;L'Intrus&lt;/em&gt; (2000), bref récit autobiographique sur sa transplantation cardiaque, mêle réflexion philosophique et expérience personnelle de la maladie et de l'altérité. Son œuvre, immense et diverse, témoigne d'une pensée vivante et rigoureuse toujours en dialogue avec la littérature, l'art et la politique. &lt;/p&gt;  &lt;audio controls title=&quot;Jean luc Nancy par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/11472-06.02.2011-ITEMA_20267545-2011C16153E0003-ITE_00040439_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" display="https://www.laphilo.fr/pho/jlnancy-mini.webp" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E132" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Philippe_Lacoue-Labarthe&quot;  title=&quot; Wikipedia&quot;&gt;Philippe LACOUE-LABARTHE&lt;/a&gt; était un philosophe, critique littéraire, traducteur et théoricien français né à Tours et connu pour ses travaux sur la mimésis, le romantisme allemand, Hölderlin, Heidegger, Derrida et la relation entre esthétique et politique. Il a aussi beaucoup compté dans le milieu intellectuel de Strasbourg, où il a enseigné longtemps et travaillé avec Jean-Luc Nancy. &lt;/p&gt; &lt;p&gt; Son  &lt;a href=&quot;https://maitron.fr/lacoue-labarthe-philippe/&quot;  title=&quot; lacoue-labarthe par le maitron&quot;&gt;œuvre interroge &lt;/a&gt; la façon dont l’art, la philosophie et la politique s’entrecroisent, notamment à travers la notion de mimésis et la critique de l’“esthétisation du politique”. Il a aussi travaillé sur le romantisme allemand et sur la réception de Hölderlin, qu’il considérait comme une figure majeure. &lt;/p&gt; &lt;p&gt; Parmi les livres souvent cités, on trouve Le Titre de la lettre avec Jean-Luc Nancy, L’Absolu littéraire, L’Imitation des modernes, La Fiction du politique et Heidegger, la politique du poème. Il a également traduit plusieurs auteurs allemands majeurs, dont Heidegger, Hölderlin, Nietzsche, Benjamin et Celan. &lt;/p&gt; &lt;p&gt; Sa pensée tourne autour de trois idées principales : - La représentation n’est jamais transparente : ce que nous montrons, racontons ou jouons n’est jamais la réalité elle-même, mais une forme, un masque, une imitation. - La littérature et le théâtre sont essentiels pour comprendre la philosophie, parce qu’ils révèlent ce que les concepts cachent ou simplifient.popups. - Le lien entre esthétique et politique est dangereux : il a beaucoup réfléchi à la manière dont l’art, les mythes et les images peuvent servir le politique, y compris dans des formes fascisantes. &lt;/p&gt; &#10; &lt;audio controls title=&quot;les versions de philippe lacoue labarthe par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/16409-16.03.2007-ITEMA_20062386-2007C6409S0011-MEM_000036772_RF-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  " r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" display="https://www.laphilo.fr/pho/pllabarthe-mini.webp" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" display="https://www.laphilo.fr/pho/fdelaporte-mini.webp" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" display="https://www.laphilo.fr/pho/lecourt-mini.webp" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E135" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Jean-Michel_Berthelot&quot;  title=&quot; Wikipedia&quot;&gt;Jean-Michel BERTHELOT&lt;/a&gt; était un philosophe et sociologue français spécialiste d'épistémologie des sciences sociales. Professeur à l'Université de Paris IV-Sorbonne et à l'Université du Québec à Montréal, il contribua de manière décisive à la réflexion philosophique sur les fondements et les méthodes des sciences humaines et sociales. Son œuvre joint la rigueur épistémologique à une large culture philosophique et sociologique. &lt;/p&gt; &lt;p&gt; Son ouvrage principal, &lt;em&gt; &lt;a href=&quot;https://www.persee.fr/doc/sotra_0038-0296_1992_num_34_3_2605_t1_0388_0000_3&quot;  title=&quot;l’intelligence du social par persée &quot;&gt; L'Intelligence du social&lt;/a&gt; &lt;/em&gt; (1990), est une analyse approfondie des schèmes d'intelligibilité que les sciences sociales utilisent pour rendre compte de la réalité sociale : le schème causal, le schème fonctionnel, le schème structural, le schème herméneutique et d'autres modes d'explication. Berthelot montre que chaque paradigme sociologique privilégie un mode d'intelligibilité particulier, ce qui permet de comprendre à la fois leurs apports spécifiques et leurs limites. Ce livre constitue l'une des contributions les plus claires et les plus systématiques à la philosophie des sciences sociales en langue française. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Epistémologie des sciences sociales&lt;/em&gt; (2001, ouvrage collectif qu'il dirigea), il offrit un panorama complet des questions épistémologiques fondamentales que posent les sciences humaines et sociales : la causalité, la compréhension, la mesure, la modélisation, la réflexivité et les rapports entre science et valeurs. Ses travaux contribuèrent à établir l'épistémologie des sciences sociales comme une discipline à part entière dans le paysage universitaire français, en dialogue constant avec la philosophie des sciences anglophones et continentale. &lt;/p&gt;" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" display="https://www.laphilo.fr/pho/jmberthelot-mini.webp" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Daniel_Bensa%C3%AFd&quot;  title=&quot; Wikipedia&quot;&gt;Daniel BENSAÏD&lt;/a&gt; était un philosophe français marxiste, l'un des intellectuels les plus importants de la gauche radicale française de son époque. Né à Paris dans une famille juive d'origine algérienne, il fut l'un des leaders de la révolte étudiante de mai 1968 à Paris-Nanterre aux côtés de Daniel Cohn-Bendit. Professeur de philosophie à l'Université Paris VIII-Saint-Denis, il fut membre dirigeant de la Ligue communiste révolutionnaire (LCR) et de son successeur le Nouveau Parti Anticapitaliste (NPA). &lt;/p&gt; &lt;p&gt; Sa pensée philosophique chercha à renouveler le marxisme en le débarrassant des &lt;a href=&quot;https://www.youtube.com/watch?v=uxBvxfRI2CE&quot;  title=&quot;la privatisation du monde par bibou11slalala &quot;&gt; simplifications téléologiques &lt;/a&gt; et en l'ouvrant à des problématiques nouvelles. Dans &lt;em&gt;Marx l'intempestif&lt;/em&gt; (1995), il défend un Marx débarrassé du déterminisme historique et de la philosophie du progrès, un Marx « intempestif » qui pense la politique comme art du possible et de l'impossible, en dialogue avec Blaise Pascal et Walter Benjamin. Ce livre renouvela profondément la  &lt;a href=&quot;https://www.youtube.com/watch?v=is8Ya038-Q4&quot;  title=&quot;l’héritage de Marx par socialtram &quot;&gt; lecture de Marx &lt;/a&gt; dans la gauche française. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Le Pari mélancolique&lt;/em&gt; (1997) et &lt;em&gt;Résistances&lt;/em&gt; (2001), il développe une philosophie de l'engagement politique nourrie par la mélancolie des défaites mais portée par une fidélité irréductible à l'émancipation. Sa réflexion sur les rapports entre philosophie et politique, entre utopie et stratégie, constitue l'une des contributions les plus originales à la pensée marxiste contemporaine. Polémiste redoutable et pédagogue exigeant, il laissa une empreinte profonde sur plusieurs générations de militants et d'intellectuels de gauche. &lt;/p&gt;  &lt;audio controls title=&quot;Daniel Bensaid  par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10075-11.12.2006-ITEMA_20049670-2006C6608S0221-MEM_000033324_RF-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; " r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" display="https://www.laphilo.fr/pho/bensaid-mini.webp" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G137" display="&quot;Ce virus est là pour nous préparer au nouveau régime climatique&quot; par France Culture" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" display="https://www.laphilo.fr/pho/latour-mini.webp" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" display="https://www.laphilo.fr/pho/rdamien-mini.webp" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Catherine_Colliot-Th%C3%A9l%C3%A8ne&quot; title=&quot; Wikipedia&quot;&gt;Catherine COLLIOT-THELENE&lt;/a&gt; était une philosophe française  majeure de la philosophie politique contemporaine, spécialiste de Max Weber et penseuse des droits, de la démocratie et de la propriété dans un cadre cosmopolitique. Membre de l’Institut universitaire de France, elle est reconnue comme une référence internationale des études wébériennes. &lt;/p&gt; &lt;p&gt; Son travail se situe au croisement de la philosophie politique et des sciences sociales, avec trois pôles principaux :  &lt;a href=&quot;https://www.youtube.com/watch?v=krUYFtq9Jww&quot; title=&quot;Max Weber et la violence légitime de l’état par France Culture&quot;&gt;Max Weber, la démocratie et les droits, &lt;/a&gt;  la propriété et le cosmopolitisme.  Elle traduit et commente plusieurs textes de Weber, notamment Le Savant et le politique et Les Communautés, en montrant en détail ses concepts de rationalisation, de désenchantement et de domination. &lt;/p&gt; &lt;p&gt; À partir des années 2000, elle se concentre sur les droits subjectifs, leur articulation avec l’individualisme contemporain et la transformation des rapports entre pouvoirs politiques et économiques. Elle insiste sur la nécessité de penser la normativité (ce qui doit être) à partir d’une analyse précise des structures sociales réelles, d’où son dialogue constant avec le droit, l’histoire et la sociologie. &lt;/p&gt; &lt;p&gt; Dans &quot;La Démocratie sans “demos”  paru en 2011, elle remet en question l’identification classique entre &quot;peuple&quot; et &quot;démocratie&quot;. Elle critique la superposition entre souveraineté du peuple et souveraineté territoriale de l’État, qui conduit selon elle à des versions exclusives de la démocratie. &lt;a href=&quot;https://www.youtube.com/watch?v=ps2ixtEpgYI&quot; title=&quot;la democratie c’est le droit de resistance par Journal l’Humanitét&quot;&gt;Sa philosophie cherche &lt;/a&gt;  une démocratie fondée sur des droits universalisables et sur la participation de tous les sujets, plutôt que sur l’appartenance à une communauté nationale préconstituée. &lt;/p&gt; &lt;p&gt; Elle refuse la séparation entre théorie pure et monde social : pour elle, la philosophie politique doit dialoguer avec les sciences sociales pour produire une critique efficace des institutions et des inégalités. Elle a accompagné, sans posture militante classique mais avec une forte implication intellectuelle, les luttes pour les droits des femmes, des exclus et des étrangers, en cherchant à fournir des outils conceptuels pour penser l’égalité aujourd’hui. &lt;/p&gt; &#10; &lt;audio controls title=&quot;Les défis juridiques de la migration : existe-t-il un droit à la libre circulation ? par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/21447-09.02.2022-ITEMA_22927630-2022C27677S0040-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" display="https://www.laphilo.fr/pho/thelene-mini.webp" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" display="https://www.laphilo.fr/pho/bstiegler-mini.webp" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bernard_Mabille_(philosophe)&quot;  style=&quot;color:#6A142A&quot;  title=&quot; Wikipedia&quot;&gt;Bernard MABILLE&lt;/a&gt; était un philosophe français spécialiste de dialectique et de philosophie hégélienne, ainsi que de métaphysique contemporaine. Agrégé de philosophie et professeur à l'Université Paris IV-Sorbonne, il fut l'un des meilleurs connaisseurs français de Hegel et contribua de manière significative au renouvellement des études hégéliennes en France dans les dernières décennies du XXe siècle. &lt;/p&gt; &lt;p&gt; Sa thèse principale, &lt;em&gt;Hegel : l'épreuve de la contingence&lt;/em&gt; (1999), est une lecture originale de la philosophie hégélienne à la lumière de la problématique de la contingence. Contre les lectures qui réduisent Hegel à un penseur du nécessaire et du rationnel, Mabille montre que la contingence est au cœur même du système hégélien et que la dialectique est précisément la méthode qui permet de penser le passage du contingent au nécessaire sans l'éliminer. Cette relecture contribua à ouvrir la philosophie hégélienne à des problématiques contemporaines. &lt;/p&gt; &lt;p&gt; Dans ses travaux sur la métaphysique et la dialectique, Mabille s'intéressa également aux rapports entre la philosophie hégélienne et la phénoménologie française, notamment Merleau-Ponty et Henry. Son enseignement à la Sorbonne forma plusieurs générations d'étudiants à la rigueur de la pensée dialectique. Sa disparition prématurée priva la philosophie française d'un penseur rigoureux dont l'œuvre, bien que de volume limité, témoigne d'une lecture profonde et originale de l'idéalisme allemand et de ses prolongements contemporains. &lt;/p&gt;" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" display="https://www.laphilo.fr/pho/bnabille-mini.webp" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" display="https://www.laphilo.fr/pho/adufourmantelle-mini.webp" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H129" display="https://www.laphilo.fr/pho/jfmarquet-mini.webp" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Cl%C3%A9ment_Rosset&quot; title=&quot; Wikipedia&quot;&gt;Clément ROSSET&lt;/a&gt; était un philosophe français connu pour sa pensée radicale et son style d'écriture d'une grande clarté. Son œuvre est principalement centrée sur le concept du  &lt;a href=&quot;https://www.youtube.com/watch?v=I50Jbj6uQEU&quot; title=&quot;Clément Rosset : la réalité ne convient pas ! par Kosmos&quot;&gt;&quot;réel&quot;&lt;/a&gt;  et l'incapacité ou la difficulté de l'homme à l'accepter dans sa singularité et souvent sa cruauté. Voici les points essentiels concernant sa philosophie : &lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.youtube.com/watch?v=8m_kXVBdtwg&quot;  title=&quot; Le réel et son double, Clément Rosset, 2.2 avant-propos par Thibault BELZACQ&quot;&gt;Le Réel sans double&lt;/a&gt; : Son idée maîtresse est que le réel est unique, singulier et dépourvu de tout &quot;double&quot;. Il n'y a pas d'arrière-monde, pas de sens caché, pas de consolation ou d'illusion qui puisse atténuer sa nature brute. Le réel est simplement ce qui est, dans son évidence la plus nue. &lt;/p&gt; &lt;p&gt; - Le Refus du double et de l'illusion : Une grande partie de son travail consiste à traquer les différentes formes d'illusions et de doubles que l'humanité crée pour  &lt;a href=&quot;https://philitt.fr/2023/09/12/clement-rosset-tout-est-sans-raison/&quot;  title=&quot;Clément Rosset : tout est sans raison par Phillitt&quot;&gt;échapper à la confrontation&lt;/a&gt; directe avec le réel. Ces doubles peuvent être d'ordre métaphysique, moral, psychologique, ou même esthétique.&lt;/p&gt; &lt;p&gt; - &lt;a href=&quot;https://www.youtube.com/watch?v=JDcudFE_uBQ&quot;  title=&quot;Entretien avec Pierre Dumayet (1961) par Archives&quot;&gt;Philosophie tragique&lt;/a&gt; et Joie : Bien que sa pensée puisse sembler sombre en insistant sur la cruauté et l'absurdité du réel, il développe une philosophie que l'on qualifie souvent de &quot;tragique&quot; au sens nietzschéen du terme. Il ne s'agit pas de désespoir, mais plutôt de l'affirmation de la vie et du réel tels qu'ils sont, y compris dans leurs aspects les plus difficiles. &lt;/p&gt; &lt;p&gt; Il est également remarquable par son style d'écriture. Loin du jargon philosophique abscons, il privilégie une langue simple, directe et percutante. Cette clarté formelle est au service de la clarté de sa pensée, cherchant à énoncer le réel avec le moins d'interférences possible. Son œuvre, bien que parfois restée en marge des courants universitaires dominants, a marqué par sa radicalité, sa lucidité et sa défense d'une confrontation sans fard avec le réel.  &lt;/p&gt; &lt;audio controls title=&quot;Clément Rosset par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10080-20.12.2013-ITEMA_20564152-2013C3403E0215-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt;&lt;/audio&gt;  " r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H130" display="https://www.laphilo.fr/pho/rosset-mini.webp" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Jacques_Bouveresse&quot;  title=&quot; Wikipedia&quot;&gt;Jacques BOUVERESSE&lt;/a&gt; était un philosophe français du courant analytique, connu pour son rationalisme exigeant, son &lt;a href=&quot;https://www.youtube.com/watch?v=mfGM00nmj20&quot;  title=&quot; Wittgenstein et l'intériorité 一 Jacques Bouveresse par Andrea Cirla &quot;&gt;travail sur Wittgenstein &lt;/a&gt; et sa critique des dérives du milieu intellectuel français. Il a largement contribué à introduire et stabiliser en France une philosophie soucieuse de vérité, de clarté et d’argumentation rigoureuse. &lt;/p&gt; &lt;p&gt; Ses domaines privilégiés sont la philosophie de la connaissance, des sciences, des mathématiques, de la logique, du langage, ainsi qu’une philosophie de la culture attentive à la littérature et à la critique sociale.  Il se réclame du rationalisme des Lumières et s’inspire fortement de la philosophie analytique, du Cercle de Vienne, de Frege, de Gödel et de la tradition d’Europe centrale. Wittgenstein, qu’il contribue à faire connaître en France, est l’une de ses références centrales. &lt;/p&gt; &lt;p&gt; Il défend une position rationaliste dont le prolongement éthique est ce qu’il appelle la  &lt;a href=&quot;https://www.persee.fr/doc/lgge_0458-726x_1971_num_6_21_2079&quot; title=&quot;Langage ordinaire et philosophie par Persée &quot;&gt;&quot;modestie intellectuelle&quot; &lt;/a&gt; : ne pas exagérer ce que la philosophie peut faire, refuser le pathos et le prestige facile. Il combat le relativisme, l’historicisme radical et les remises en cause globales de la notion de vérité, notamment chez certains auteurs français, tout en reconnaissant par ailleurs leur importance. &lt;/p&gt; &lt;p&gt; Sa grande thèse, &quot;Le Mythe de l’intériorité&quot;, porte sur Wittgenstein, le langage privé, l’expérience et la signification, et a joué un rôle clé dans la réception française de Wittgenstein. Il consacre de nombreux travaux à Robert Musil et Karl Kraus, qu’il lit comme des alliés dans un combat pour l’exactitude, la critique de la bêtise et des illusions de la culture moderne. &lt;/p&gt;  &lt;audio controls title=&quot;Jacques Bouveresse, à la recherche de la clarté par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10351-11.05.2021-ITEMA_23961779-2000C3500E0287-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H131" display="https://www.laphilo.fr/pho/bouveresse-mini.webp" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E132" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Jean-Luc_Nancy&quot;  title=&quot; Wikipedia&quot;&gt;Jean-Luc NANCY&lt;/a&gt; était un philosophe français, agrégé de philosophie, il fut professeur à l'Université de Strasbourg jusqu'à sa retraite. Sa pensée, en dialogue constant avec Heidegger, Derrida et Lacoue-Labarthe — avec lequel il collabora étroitement — porte sur le « sens du monde », la communauté, le corps et le toucher. &lt;/p&gt; &lt;p&gt; Son œuvre est marquée par le questionnement du « with » (avec), du « being-with » heideggerien. Dans &lt;em&gt;La Communauté désoeuvrée&lt;/em&gt; (1986), il développe une pensée de la communauté qui refuse toute forme d'immanentisme ou de fusion : la communauté véritable n'est pas une substance commune, mais  &lt;a href=&quot;https://www.youtube.com/watch?v=fZK6pEAPxEw&quot;  title=&quot;jean luc Nancy par Institut Humanités &quot;&gt;l'exposition partagée &lt;/a&gt; de la singularité de chacun. Cette réflexion, en dialogue critique avec Blanchot et Bataille, a eu un retentissement considérable dans les débats contemporains sur la politique, la communauté et l'identité. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Corpus&lt;/em&gt; (1992) et &lt;em&gt;Noli me tangere&lt;/em&gt; (2003), il explore  &lt;a href=&quot;https://www.youtube.com/watch?v=1kCExw6Wp9k&quot;  title=&quot;jean luc Nancy par Lacan TV &quot;&gt;la philosophie du corps &lt;/a&gt; et du toucher comme modes fondamentaux de l'être-au-monde. Son essai sur le sens — &lt;em&gt;Le Sens du monde&lt;/em&gt; (1993) — aborde la question de la possibilité du sens dans un monde déserté par les transcendances. &lt;em&gt;L'Intrus&lt;/em&gt; (2000), bref récit autobiographique sur sa transplantation cardiaque, mêle réflexion philosophique et expérience personnelle de la maladie et de l'altérité. Son œuvre, immense et diverse, témoigne d'une pensée vivante et rigoureuse toujours en dialogue avec la littérature, l'art et la politique. &lt;/p&gt;  &lt;audio controls title=&quot;Jean luc Nancy par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/11472-06.02.2011-ITEMA_20267545-2011C16153E0003-ITE_00040439_RSCE-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H132" display="https://www.laphilo.fr/pho/jlnancy-mini.webp" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E133" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Philippe_Lacoue-Labarthe&quot;  title=&quot; Wikipedia&quot;&gt;Philippe LACOUE-LABARTHE&lt;/a&gt; était un philosophe, critique littéraire, traducteur et théoricien français né à Tours et connu pour ses travaux sur la mimésis, le romantisme allemand, Hölderlin, Heidegger, Derrida et la relation entre esthétique et politique. Il a aussi beaucoup compté dans le milieu intellectuel de Strasbourg, où il a enseigné longtemps et travaillé avec Jean-Luc Nancy. &lt;/p&gt; &lt;p&gt; Son  &lt;a href=&quot;https://maitron.fr/lacoue-labarthe-philippe/&quot;  title=&quot; lacoue-labarthe par le maitron&quot;&gt;œuvre interroge &lt;/a&gt; la façon dont l’art, la philosophie et la politique s’entrecroisent, notamment à travers la notion de mimésis et la critique de l’“esthétisation du politique”. Il a aussi travaillé sur le romantisme allemand et sur la réception de Hölderlin, qu’il considérait comme une figure majeure. &lt;/p&gt; &lt;p&gt; Parmi les livres souvent cités, on trouve Le Titre de la lettre avec Jean-Luc Nancy, L’Absolu littéraire, L’Imitation des modernes, La Fiction du politique et Heidegger, la politique du poème. Il a également traduit plusieurs auteurs allemands majeurs, dont Heidegger, Hölderlin, Nietzsche, Benjamin et Celan. &lt;/p&gt; &lt;p&gt; Sa pensée tourne autour de trois idées principales : - La représentation n’est jamais transparente : ce que nous montrons, racontons ou jouons n’est jamais la réalité elle-même, mais une forme, un masque, une imitation. - La littérature et le théâtre sont essentiels pour comprendre la philosophie, parce qu’ils révèlent ce que les concepts cachent ou simplifient.popups. - Le lien entre esthétique et politique est dangereux : il a beaucoup réfléchi à la manière dont l’art, les mythes et les images peuvent servir le politique, y compris dans des formes fascisantes. &lt;/p&gt; &#10; &lt;audio controls title=&quot;les versions de philippe lacoue labarthe par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/16409-16.03.2007-ITEMA_20062386-2007C6409S0011-MEM_000036772_RF-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;  " r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H133" display="https://www.laphilo.fr/pho/pllabarthe-mini.webp" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H134" display="https://www.laphilo.fr/pho/fdelaporte-mini.webp" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H135" display="https://www.laphilo.fr/pho/lecourt-mini.webp" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Jean-Michel_Berthelot&quot;  title=&quot; Wikipedia&quot;&gt;Jean-Michel BERTHELOT&lt;/a&gt; était un philosophe et sociologue français spécialiste d'épistémologie des sciences sociales. Professeur à l'Université de Paris IV-Sorbonne et à l'Université du Québec à Montréal, il contribua de manière décisive à la réflexion philosophique sur les fondements et les méthodes des sciences humaines et sociales. Son œuvre joint la rigueur épistémologique à une large culture philosophique et sociologique. &lt;/p&gt; &lt;p&gt; Son ouvrage principal, &lt;em&gt; &lt;a href=&quot;https://www.persee.fr/doc/sotra_0038-0296_1992_num_34_3_2605_t1_0388_0000_3&quot;  title=&quot;l’intelligence du social par persée &quot;&gt; L'Intelligence du social&lt;/a&gt; &lt;/em&gt; (1990), est une analyse approfondie des schèmes d'intelligibilité que les sciences sociales utilisent pour rendre compte de la réalité sociale : le schème causal, le schème fonctionnel, le schème structural, le schème herméneutique et d'autres modes d'explication. Berthelot montre que chaque paradigme sociologique privilégie un mode d'intelligibilité particulier, ce qui permet de comprendre à la fois leurs apports spécifiques et leurs limites. Ce livre constitue l'une des contributions les plus claires et les plus systématiques à la philosophie des sciences sociales en langue française. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Epistémologie des sciences sociales&lt;/em&gt; (2001, ouvrage collectif qu'il dirigea), il offrit un panorama complet des questions épistémologiques fondamentales que posent les sciences humaines et sociales : la causalité, la compréhension, la mesure, la modélisation, la réflexivité et les rapports entre science et valeurs. Ses travaux contribuèrent à établir l'épistémologie des sciences sociales comme une discipline à part entière dans le paysage universitaire français, en dialogue constant avec la philosophie des sciences anglophones et continentale. &lt;/p&gt;" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H136" display="https://www.laphilo.fr/pho/jmberthelot-mini.webp" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Daniel_Bensa%C3%AFd&quot;  title=&quot; Wikipedia&quot;&gt;Daniel BENSAÏD&lt;/a&gt; était un philosophe français marxiste, l'un des intellectuels les plus importants de la gauche radicale française de son époque. Né à Paris dans une famille juive d'origine algérienne, il fut l'un des leaders de la révolte étudiante de mai 1968 à Paris-Nanterre aux côtés de Daniel Cohn-Bendit. Professeur de philosophie à l'Université Paris VIII-Saint-Denis, il fut membre dirigeant de la Ligue communiste révolutionnaire (LCR) et de son successeur le Nouveau Parti Anticapitaliste (NPA). &lt;/p&gt; &lt;p&gt; Sa pensée philosophique chercha à renouveler le marxisme en le débarrassant des &lt;a href=&quot;https://www.youtube.com/watch?v=uxBvxfRI2CE&quot;  title=&quot;la privatisation du monde par bibou11slalala &quot;&gt; simplifications téléologiques &lt;/a&gt; et en l'ouvrant à des problématiques nouvelles. Dans &lt;em&gt;Marx l'intempestif&lt;/em&gt; (1995), il défend un Marx débarrassé du déterminisme historique et de la philosophie du progrès, un Marx « intempestif » qui pense la politique comme art du possible et de l'impossible, en dialogue avec Blaise Pascal et Walter Benjamin. Ce livre renouvela profondément la  &lt;a href=&quot;https://www.youtube.com/watch?v=is8Ya038-Q4&quot;  title=&quot;l’héritage de Marx par socialtram &quot;&gt; lecture de Marx &lt;/a&gt; dans la gauche française. &lt;/p&gt; &lt;p&gt; Dans &lt;em&gt;Le Pari mélancolique&lt;/em&gt; (1997) et &lt;em&gt;Résistances&lt;/em&gt; (2001), il développe une philosophie de l'engagement politique nourrie par la mélancolie des défaites mais portée par une fidélité irréductible à l'émancipation. Sa réflexion sur les rapports entre philosophie et politique, entre utopie et stratégie, constitue l'une des contributions les plus originales à la pensée marxiste contemporaine. Polémiste redoutable et pédagogue exigeant, il laissa une empreinte profonde sur plusieurs générations de militants et d'intellectuels de gauche. &lt;/p&gt;  &lt;audio controls title=&quot;Daniel Bensaid  par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/10075-11.12.2006-ITEMA_20049670-2006C6608S0221-MEM_000033324_RF-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt; " r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H137" display="https://www.laphilo.fr/pho/bensaid-mini.webp" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G138" display="&quot;Ce virus est là pour nous préparer au nouveau régime climatique&quot; par France Culture" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H138" display="https://www.laphilo.fr/pho/latour-mini.webp" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H139" display="https://www.laphilo.fr/pho/rdamien-mini.webp" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Catherine_Colliot-Th%C3%A9l%C3%A8ne&quot; title=&quot; Wikipedia&quot;&gt;Catherine COLLIOT-THELENE&lt;/a&gt; était une philosophe française  majeure de la philosophie politique contemporaine, spécialiste de Max Weber et penseuse des droits, de la démocratie et de la propriété dans un cadre cosmopolitique. Membre de l’Institut universitaire de France, elle est reconnue comme une référence internationale des études wébériennes. &lt;/p&gt; &lt;p&gt; Son travail se situe au croisement de la philosophie politique et des sciences sociales, avec trois pôles principaux :  &lt;a href=&quot;https://www.youtube.com/watch?v=krUYFtq9Jww&quot; title=&quot;Max Weber et la violence légitime de l’état par France Culture&quot;&gt;Max Weber, la démocratie et les droits, &lt;/a&gt;  la propriété et le cosmopolitisme.  Elle traduit et commente plusieurs textes de Weber, notamment Le Savant et le politique et Les Communautés, en montrant en détail ses concepts de rationalisation, de désenchantement et de domination. &lt;/p&gt; &lt;p&gt; À partir des années 2000, elle se concentre sur les droits subjectifs, leur articulation avec l’individualisme contemporain et la transformation des rapports entre pouvoirs politiques et économiques. Elle insiste sur la nécessité de penser la normativité (ce qui doit être) à partir d’une analyse précise des structures sociales réelles, d’où son dialogue constant avec le droit, l’histoire et la sociologie. &lt;/p&gt; &lt;p&gt; Dans &quot;La Démocratie sans “demos”  paru en 2011, elle remet en question l’identification classique entre &quot;peuple&quot; et &quot;démocratie&quot;. Elle critique la superposition entre souveraineté du peuple et souveraineté territoriale de l’État, qui conduit selon elle à des versions exclusives de la démocratie. &lt;a href=&quot;https://www.youtube.com/watch?v=ps2ixtEpgYI&quot; title=&quot;la democratie c’est le droit de resistance par Journal l’Humanitét&quot;&gt;Sa philosophie cherche &lt;/a&gt;  une démocratie fondée sur des droits universalisables et sur la participation de tous les sujets, plutôt que sur l’appartenance à une communauté nationale préconstituée. &lt;/p&gt; &lt;p&gt; Elle refuse la séparation entre théorie pure et monde social : pour elle, la philosophie politique doit dialoguer avec les sciences sociales pour produire une critique efficace des institutions et des inégalités. Elle a accompagné, sans posture militante classique mais avec une forte implication intellectuelle, les luttes pour les droits des femmes, des exclus et des étrangers, en cherchant à fournir des outils conceptuels pour penser l’égalité aujourd’hui. &lt;/p&gt; &#10; &lt;audio controls title=&quot;Les défis juridiques de la migration : existe-t-il un droit à la libre circulation ? par France Culture&quot;&gt; &lt;source src=&quot;https://media.radiofrance-podcast.net/podcast09/21447-09.02.2022-ITEMA_22927630-2022C27677S0040-21.mp3&quot; type=&quot;audio/mpeg&quot; align=&quot;center&quot;&gt; &lt;/audio&gt;" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H140" display="https://www.laphilo.fr/pho/thelene-mini.webp" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H141" display="https://www.laphilo.fr/pho/bstiegler-mini.webp" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" display="&lt;p&gt;&lt;a href=&quot;https://fr.wikipedia.org/wiki/Bernard_Mabille_(philosophe)&quot;  style=&quot;color:#6A142A&quot;  title=&quot; Wikipedia&quot;&gt;Bernard MABILLE&lt;/a&gt; était un philosophe français spécialiste de dialectique et de philosophie hégélienne, ainsi que de métaphysique contemporaine. Agrégé de philosophie et professeur à l'Université Paris IV-Sorbonne, il fut l'un des meilleurs connaisseurs français de Hegel et contribua de manière significative au renouvellement des études hégéliennes en France dans les dernières décennies du XXe siècle. &lt;/p&gt; &lt;p&gt; Sa thèse principale, &lt;em&gt;Hegel : l'épreuve de la contingence&lt;/em&gt; (1999), est une lecture originale de la philosophie hégélienne à la lumière de la problématique de la contingence. Contre les lectures qui réduisent Hegel à un penseur du nécessaire et du rationnel, Mabille montre que la contingence est au cœur même du système hégélien et que la dialectique est précisément la méthode qui permet de penser le passage du contingent au nécessaire sans l'éliminer. Cette relecture contribua à ouvrir la philosophie hégélienne à des problématiques contemporaines. &lt;/p&gt; &lt;p&gt; Dans ses travaux sur la métaphysique et la dialectique, Mabille s'intéressa également aux rapports entre la philosophie hégélienne et la phénoménologie française, notamment Merleau-Ponty et Henry. Son enseignement à la Sorbonne forma plusieurs générations d'étudiants à la rigueur de la pensée dialectique. Sa disparition prématurée priva la philosophie française d'un penseur rigoureux dont l'œuvre, bien que de volume limité, témoigne d'une lecture profonde et originale de l'idéalisme allemand et de ses prolongements contemporains. &lt;/p&gt;" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H142" display="https://www.laphilo.fr/pho/bnabille-mini.webp" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H143" display="https://www.laphilo.fr/pho/adufourmantelle-mini.webp" r:id="rId105"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>